<commit_message>
Pack v2: nine working tabs and the Inspection Playbook
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pack/staffbook-staff-file-pack.xlsx
+++ b/pack/staffbook-staff-file-pack.xlsx
@@ -4,16 +4,24 @@
   <sheets>
     <sheet name="Training matrix" sheetId="1" r:id="rId1"/>
     <sheet name="Expiries (automatic)" sheetId="2" r:id="rId2"/>
-    <sheet name="Staff file checklist" sheetId="3" r:id="rId3"/>
-    <sheet name="Employment gaps" sheetId="4" r:id="rId4"/>
-    <sheet name="Inspection self-audit" sheetId="5" r:id="rId5"/>
+    <sheet name="Supervision tracker" sheetId="3" r:id="rId3"/>
+    <sheet name="DBS re-check log" sheetId="4" r:id="rId4"/>
+    <sheet name="Diploma clocks" sheetId="5" r:id="rId5"/>
+    <sheet name="Governance clocks" sheetId="6" r:id="rId6"/>
+    <sheet name="Staff file checklist" sheetId="7" r:id="rId7"/>
+    <sheet name="Employment gaps" sheetId="8" r:id="rId8"/>
+    <sheet name="Inspection self-audit" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Training matrix'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Expiries (automatic)'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Staff file checklist'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Employment gaps'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Inspection self-audit'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Supervision tracker'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'DBS re-check log'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Diploma clocks'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Governance clocks'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Staff file checklist'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Employment gaps'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Inspection self-audit'!$4:$4</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -86,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1"/>
@@ -99,6 +107,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyFont="1" applyFill="1"/>
@@ -170,7 +181,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Type each completion date under the course. The Expiries tab colours itself: red has run out, amber is due within 30 days. Given free by Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
+          <t>Type each completion date under the course. The Expiries tab does the rest. Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
         </is>
       </c>
     </row>
@@ -328,7 +339,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nothing to type here. Red has expired, amber is due within 30 days, green is in date.</t>
+          <t>Nothing to type here. Red has expired, amber is due within 30 days, green is fine. Check it every Monday.</t>
         </is>
       </c>
     </row>
@@ -1036,6 +1047,1043 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Supervision tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Name, your cycle in days (28 is common), and the date of the last supervision. The rest computes itself. The manager goes on this list too: theirs is the record inspectors ask for first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Staff member</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Cycle (days)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Last supervision</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Days since</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Standing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Example: change or delete this row</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <v>28</v>
+      </c>
+      <c r="C5" s="7">
+        <v>46219</v>
+      </c>
+      <c r="D5" s="8">
+        <f>IF(C5="","",TODAY()-C5)</f>
+      </c>
+      <c r="E5" s="8">
+        <f>IF(C5="","",IF(TODAY()-C5&gt;B5,"OVERDUE",IF(TODAY()-C5&gt;B5-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="8">
+        <v>28</v>
+      </c>
+      <c r="D6" s="8">
+        <f>IF(C6="","",TODAY()-C6)</f>
+      </c>
+      <c r="E6" s="8">
+        <f>IF(C6="","",IF(TODAY()-C6&gt;B6,"OVERDUE",IF(TODAY()-C6&gt;B6-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="8">
+        <v>28</v>
+      </c>
+      <c r="D7" s="8">
+        <f>IF(C7="","",TODAY()-C7)</f>
+      </c>
+      <c r="E7" s="8">
+        <f>IF(C7="","",IF(TODAY()-C7&gt;B7,"OVERDUE",IF(TODAY()-C7&gt;B7-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="8">
+        <v>28</v>
+      </c>
+      <c r="D8" s="8">
+        <f>IF(C8="","",TODAY()-C8)</f>
+      </c>
+      <c r="E8" s="8">
+        <f>IF(C8="","",IF(TODAY()-C8&gt;B8,"OVERDUE",IF(TODAY()-C8&gt;B8-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="8">
+        <v>28</v>
+      </c>
+      <c r="D9" s="8">
+        <f>IF(C9="","",TODAY()-C9)</f>
+      </c>
+      <c r="E9" s="8">
+        <f>IF(C9="","",IF(TODAY()-C9&gt;B9,"OVERDUE",IF(TODAY()-C9&gt;B9-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="8">
+        <v>28</v>
+      </c>
+      <c r="D10" s="8">
+        <f>IF(C10="","",TODAY()-C10)</f>
+      </c>
+      <c r="E10" s="8">
+        <f>IF(C10="","",IF(TODAY()-C10&gt;B10,"OVERDUE",IF(TODAY()-C10&gt;B10-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="8">
+        <v>28</v>
+      </c>
+      <c r="D11" s="8">
+        <f>IF(C11="","",TODAY()-C11)</f>
+      </c>
+      <c r="E11" s="8">
+        <f>IF(C11="","",IF(TODAY()-C11&gt;B11,"OVERDUE",IF(TODAY()-C11&gt;B11-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="8">
+        <v>28</v>
+      </c>
+      <c r="D12" s="8">
+        <f>IF(C12="","",TODAY()-C12)</f>
+      </c>
+      <c r="E12" s="8">
+        <f>IF(C12="","",IF(TODAY()-C12&gt;B12,"OVERDUE",IF(TODAY()-C12&gt;B12-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="8">
+        <v>28</v>
+      </c>
+      <c r="D13" s="8">
+        <f>IF(C13="","",TODAY()-C13)</f>
+      </c>
+      <c r="E13" s="8">
+        <f>IF(C13="","",IF(TODAY()-C13&gt;B13,"OVERDUE",IF(TODAY()-C13&gt;B13-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="8">
+        <v>28</v>
+      </c>
+      <c r="D14" s="8">
+        <f>IF(C14="","",TODAY()-C14)</f>
+      </c>
+      <c r="E14" s="8">
+        <f>IF(C14="","",IF(TODAY()-C14&gt;B14,"OVERDUE",IF(TODAY()-C14&gt;B14-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="8">
+        <v>28</v>
+      </c>
+      <c r="D15" s="8">
+        <f>IF(C15="","",TODAY()-C15)</f>
+      </c>
+      <c r="E15" s="8">
+        <f>IF(C15="","",IF(TODAY()-C15&gt;B15,"OVERDUE",IF(TODAY()-C15&gt;B15-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="8">
+        <v>28</v>
+      </c>
+      <c r="D16" s="8">
+        <f>IF(C16="","",TODAY()-C16)</f>
+      </c>
+      <c r="E16" s="8">
+        <f>IF(C16="","",IF(TODAY()-C16&gt;B16,"OVERDUE",IF(TODAY()-C16&gt;B16-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8">
+        <v>28</v>
+      </c>
+      <c r="D17" s="8">
+        <f>IF(C17="","",TODAY()-C17)</f>
+      </c>
+      <c r="E17" s="8">
+        <f>IF(C17="","",IF(TODAY()-C17&gt;B17,"OVERDUE",IF(TODAY()-C17&gt;B17-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="8">
+        <v>28</v>
+      </c>
+      <c r="D18" s="8">
+        <f>IF(C18="","",TODAY()-C18)</f>
+      </c>
+      <c r="E18" s="8">
+        <f>IF(C18="","",IF(TODAY()-C18&gt;B18,"OVERDUE",IF(TODAY()-C18&gt;B18-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="8">
+        <v>28</v>
+      </c>
+      <c r="D19" s="8">
+        <f>IF(C19="","",TODAY()-C19)</f>
+      </c>
+      <c r="E19" s="8">
+        <f>IF(C19="","",IF(TODAY()-C19&gt;B19,"OVERDUE",IF(TODAY()-C19&gt;B19-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="8">
+        <v>28</v>
+      </c>
+      <c r="D20" s="8">
+        <f>IF(C20="","",TODAY()-C20)</f>
+      </c>
+      <c r="E20" s="8">
+        <f>IF(C20="","",IF(TODAY()-C20&gt;B20,"OVERDUE",IF(TODAY()-C20&gt;B20-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="8">
+        <v>28</v>
+      </c>
+      <c r="D21" s="8">
+        <f>IF(C21="","",TODAY()-C21)</f>
+      </c>
+      <c r="E21" s="8">
+        <f>IF(C21="","",IF(TODAY()-C21&gt;B21,"OVERDUE",IF(TODAY()-C21&gt;B21-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="8">
+        <v>28</v>
+      </c>
+      <c r="D22" s="8">
+        <f>IF(C22="","",TODAY()-C22)</f>
+      </c>
+      <c r="E22" s="8">
+        <f>IF(C22="","",IF(TODAY()-C22&gt;B22,"OVERDUE",IF(TODAY()-C22&gt;B22-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="8">
+        <v>28</v>
+      </c>
+      <c r="D23" s="8">
+        <f>IF(C23="","",TODAY()-C23)</f>
+      </c>
+      <c r="E23" s="8">
+        <f>IF(C23="","",IF(TODAY()-C23&gt;B23,"OVERDUE",IF(TODAY()-C23&gt;B23-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="8">
+        <v>28</v>
+      </c>
+      <c r="D24" s="8">
+        <f>IF(C24="","",TODAY()-C24)</f>
+      </c>
+      <c r="E24" s="8">
+        <f>IF(C24="","",IF(TODAY()-C24&gt;B24,"OVERDUE",IF(TODAY()-C24&gt;B24-7,"DUE","OK")))</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="8">
+        <v>28</v>
+      </c>
+      <c r="D25" s="8">
+        <f>IF(C25="","",TODAY()-C25)</f>
+      </c>
+      <c r="E25" s="8">
+        <f>IF(C25="","",IF(TODAY()-C25&gt;B25,"OVERDUE",IF(TODAY()-C25&gt;B25-7,"DUE","OK")))</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E5:E25">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>E5="OVERDUE"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>E5="DUE"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>E5="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF0D5C45"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DBS re-check log</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>For staff on the Update Service: run the status check twice a year (one minute each, with consent) and note the date. Next due computes itself. "When did you last check?" is a real inspection question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Staff member</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Certificate number</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>On the Update Service?</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Last status check</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Next check due</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Example: change or delete this row</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>001234567890</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" s="7">
+        <v>46059</v>
+      </c>
+      <c r="E5" s="7">
+        <f>IF(D5="","",EDATE(D5,6))</f>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>No change</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="E6" s="7">
+        <f>IF(D6="","",EDATE(D6,6))</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7" s="7">
+        <f>IF(D7="","",EDATE(D7,6))</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="E8" s="7">
+        <f>IF(D8="","",EDATE(D8,6))</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="E9" s="7">
+        <f>IF(D9="","",EDATE(D9,6))</f>
+      </c>
+    </row>
+    <row r="10">
+      <c r="E10" s="7">
+        <f>IF(D10="","",EDATE(D10,6))</f>
+      </c>
+    </row>
+    <row r="11">
+      <c r="E11" s="7">
+        <f>IF(D11="","",EDATE(D11,6))</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" s="7">
+        <f>IF(D12="","",EDATE(D12,6))</f>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" s="7">
+        <f>IF(D13="","",EDATE(D13,6))</f>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" s="7">
+        <f>IF(D14="","",EDATE(D14,6))</f>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" s="7">
+        <f>IF(D15="","",EDATE(D15,6))</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="7">
+        <f>IF(D16="","",EDATE(D16,6))</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="7">
+        <f>IF(D17="","",EDATE(D17,6))</f>
+      </c>
+    </row>
+    <row r="18">
+      <c r="E18" s="7">
+        <f>IF(D18="","",EDATE(D18,6))</f>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" s="7">
+        <f>IF(D19="","",EDATE(D19,6))</f>
+      </c>
+    </row>
+    <row r="20">
+      <c r="E20" s="7">
+        <f>IF(D20="","",EDATE(D20,6))</f>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" s="7">
+        <f>IF(D21="","",EDATE(D21,6))</f>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" s="7">
+        <f>IF(D22="","",EDATE(D22,6))</f>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" s="7">
+        <f>IF(D23="","",EDATE(D23,6))</f>
+      </c>
+    </row>
+    <row r="24">
+      <c r="E24" s="7">
+        <f>IF(D24="","",EDATE(D24,6))</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" s="7">
+        <f>IF(D25="","",EDATE(D25,6))</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E5:E25">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(E5&lt;&gt;"",E5&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>AND(E5&lt;&gt;"",E5&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>AND(E5&lt;&gt;"",E5&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF0D5C45"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Diploma clocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Care staff must gain the Level 3 Diploma within two years of starting. Type their start date and whether they hold it; the deadline computes itself and goes red when it passes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Staff member</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Start date</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Holds Level 3? (Yes/No)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Level 3 due by</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Example: change or delete this row</t>
+        </is>
+      </c>
+      <c r="B5" s="7">
+        <v>45759</v>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" s="7">
+        <f>IF(OR(B5="",C5="Yes"),"",EDATE(B5,24))</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="8"/>
+      <c r="D6" s="7">
+        <f>IF(OR(B6="",C6="Yes"),"",EDATE(B6,24))</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" s="8"/>
+      <c r="D7" s="7">
+        <f>IF(OR(B7="",C7="Yes"),"",EDATE(B7,24))</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="8"/>
+      <c r="D8" s="7">
+        <f>IF(OR(B8="",C8="Yes"),"",EDATE(B8,24))</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="8"/>
+      <c r="D9" s="7">
+        <f>IF(OR(B9="",C9="Yes"),"",EDATE(B9,24))</f>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="8"/>
+      <c r="D10" s="7">
+        <f>IF(OR(B10="",C10="Yes"),"",EDATE(B10,24))</f>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="8"/>
+      <c r="D11" s="7">
+        <f>IF(OR(B11="",C11="Yes"),"",EDATE(B11,24))</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="8"/>
+      <c r="D12" s="7">
+        <f>IF(OR(B12="",C12="Yes"),"",EDATE(B12,24))</f>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="8"/>
+      <c r="D13" s="7">
+        <f>IF(OR(B13="",C13="Yes"),"",EDATE(B13,24))</f>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="8"/>
+      <c r="D14" s="7">
+        <f>IF(OR(B14="",C14="Yes"),"",EDATE(B14,24))</f>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="8"/>
+      <c r="D15" s="7">
+        <f>IF(OR(B15="",C15="Yes"),"",EDATE(B15,24))</f>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" s="8"/>
+      <c r="D16" s="7">
+        <f>IF(OR(B16="",C16="Yes"),"",EDATE(B16,24))</f>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="8"/>
+      <c r="D17" s="7">
+        <f>IF(OR(B17="",C17="Yes"),"",EDATE(B17,24))</f>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="8"/>
+      <c r="D18" s="7">
+        <f>IF(OR(B18="",C18="Yes"),"",EDATE(B18,24))</f>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="8"/>
+      <c r="D19" s="7">
+        <f>IF(OR(B19="",C19="Yes"),"",EDATE(B19,24))</f>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="8"/>
+      <c r="D20" s="7">
+        <f>IF(OR(B20="",C20="Yes"),"",EDATE(B20,24))</f>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="8"/>
+      <c r="D21" s="7">
+        <f>IF(OR(B21="",C21="Yes"),"",EDATE(B21,24))</f>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="8"/>
+      <c r="D22" s="7">
+        <f>IF(OR(B22="",C22="Yes"),"",EDATE(B22,24))</f>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" s="8"/>
+      <c r="D23" s="7">
+        <f>IF(OR(B23="",C23="Yes"),"",EDATE(B23,24))</f>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="8"/>
+      <c r="D24" s="7">
+        <f>IF(OR(B24="",C24="Yes"),"",EDATE(B24,24))</f>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="8"/>
+      <c r="D25" s="7">
+        <f>IF(OR(B25="",C25="Yes"),"",EDATE(B25,24))</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D25">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(D5&lt;&gt;"",D5&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>AND(D5&lt;&gt;"",D5&lt;TODAY()+90)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>AND(D5&lt;&gt;"",D5&gt;=TODAY()+90)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF0D5C45"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Governance clocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The documents every home must keep under review. Type the date each was last reviewed; the next-due date computes itself. Below: the two visit clocks inspectors always check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Last reviewed</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Review every (months)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Next due</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Statement of purpose</t>
+        </is>
+      </c>
+      <c r="C5" s="8">
+        <v>12</v>
+      </c>
+      <c r="D5" s="7">
+        <f>IF(B5="","",EDATE(B5,C5))</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Location risk assessment</t>
+        </is>
+      </c>
+      <c r="C6" s="8">
+        <v>12</v>
+      </c>
+      <c r="D6" s="7">
+        <f>IF(B6="","",EDATE(B6,C6))</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Safeguarding policy</t>
+        </is>
+      </c>
+      <c r="C7" s="8">
+        <v>12</v>
+      </c>
+      <c r="D7" s="7">
+        <f>IF(B7="","",EDATE(B7,C7))</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Behaviour support policy</t>
+        </is>
+      </c>
+      <c r="C8" s="8">
+        <v>12</v>
+      </c>
+      <c r="D8" s="7">
+        <f>IF(B8="","",EDATE(B8,C8))</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Missing child policy</t>
+        </is>
+      </c>
+      <c r="C9" s="8">
+        <v>12</v>
+      </c>
+      <c r="D9" s="7">
+        <f>IF(B9="","",EDATE(B9,C9))</f>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Complaints policy</t>
+        </is>
+      </c>
+      <c r="C10" s="8">
+        <v>12</v>
+      </c>
+      <c r="D10" s="7">
+        <f>IF(B10="","",EDATE(B10,C10))</f>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lone working assessment</t>
+        </is>
+      </c>
+      <c r="C11" s="8">
+        <v>12</v>
+      </c>
+      <c r="D11" s="7">
+        <f>IF(B11="","",EDATE(B11,C11))</f>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Workforce plan</t>
+        </is>
+      </c>
+      <c r="C12" s="8">
+        <v>12</v>
+      </c>
+      <c r="D12" s="7">
+        <f>IF(B12="","",EDATE(B12,C12))</f>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>The two visit clocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Reg 44 visit date</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Report received</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Actions all closed?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>February</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>March</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>June</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>July</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>August</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>October</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>December</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Reg 45 quality of care review: due every six months, sent to Ofsted within 28 days of completing it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D12">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(D5&lt;&gt;"",D5&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>AND(D5&lt;&gt;"",D5&lt;TODAY()+60)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>AND(D5&lt;&gt;"",D5&gt;=TODAY()+60)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF0D5C45"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -1098,19 +2146,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Enhanced DBS with children's barred list check</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Certificate number and date recorded; the disclosure content itself is never filed</t>
-        </is>
-      </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Certificate number and date recorded; never the disclosure content</t>
+        </is>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1120,24 +2168,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>On file, verified by phone, with a note of the call</t>
+          <t>On file, checked by phone, with a note of the call</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Why previous work with children or vulnerable adults ended</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Verified so far as practicable, in writing</t>
-        </is>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Checked as far as practicable, in writing</t>
+        </is>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1152,19 +2200,19 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Full employment history with every gap explained in writing</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Use the Employment gaps tab; anything over a month needs an explanation</t>
-        </is>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Use the Employment gaps tab; anything over a month needs a sentence</t>
+        </is>
+      </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1179,19 +2227,19 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Health: mentally and physically fit for the role</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Assessment date recorded; keep the assessment itself with occupational health</t>
-        </is>
-      </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Health: fit for the role</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Assessment date recorded; the assessment itself stays with occupational health</t>
+        </is>
+      </c>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1206,19 +2254,19 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>DBS Update Service status, if subscribed</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Consent noted and the date of the last status check</t>
         </is>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1230,7 +2278,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0D5C45"/>
@@ -1256,7 +2304,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Work backwards from their current job. The single most common file failure is a gap with no written explanation; "travelling" or "not working" written down is a pass, silence is a finding.</t>
+          <t>Work backwards from their current job. The most common file failure is a gap with no written explanation. "Travelling" written down is a pass. Silence is a finding.</t>
         </is>
       </c>
     </row>
@@ -1289,72 +2337,72 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Verified?</t>
+          <t>Checked?</t>
         </is>
       </c>
     </row>
     <row r="5"/>
     <row r="6">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7"/>
     <row r="8">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11"/>
     <row r="12">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
     </row>
     <row r="15"/>
     <row r="16">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
     </row>
     <row r="17"/>
     <row r="18">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
     </row>
     <row r="19"/>
   </sheetData>
@@ -1367,7 +2415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF0D5C45"/>
@@ -1391,7 +2439,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The eleven staff-side things every full inspection asks for (SCCIF Annex A). Grade yourself honestly before Ofsted does it for you.</t>
+          <t>The eleven staff-side things every full inspection asks for. Grade yourself honestly before Ofsted does it for you.</t>
         </is>
       </c>
     </row>
@@ -1426,14 +2474,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Staff list with qualifications and planned qualification updates</t>
         </is>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1443,14 +2491,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Training records, mandatory courses in date</t>
         </is>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1460,14 +2508,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Staffing rotas, planned and as actually worked</t>
         </is>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1477,14 +2525,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Reports of monthly regulation 44 visits</t>
         </is>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1494,14 +2542,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Notifications made to Ofsted, with who else was told</t>
         </is>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1514,7 +2562,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Given free by Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
+          <t>Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pack v3: instant-feedback matrix and a Start here tab
Colby typed a date and nothing visibly happened, because the result
lived on a second tab and the renews-every row looked like a data
row. One tab now: Done on next to Expires (auto) per course, the
expiry fills in and colours itself the moment a date lands, renewal
info lives in the course header, and a Start here tab explains every
tab in a minute. Example rows show all three colours live.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pack/staffbook-staff-file-pack.xlsx
+++ b/pack/staffbook-staff-file-pack.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Training matrix" sheetId="1" r:id="rId1"/>
-    <sheet name="Expiries (automatic)" sheetId="2" r:id="rId2"/>
+    <sheet name="Start here" sheetId="1" r:id="rId1"/>
+    <sheet name="Training matrix" sheetId="2" r:id="rId2"/>
     <sheet name="Supervision tracker" sheetId="3" r:id="rId3"/>
     <sheet name="DBS re-check log" sheetId="4" r:id="rId4"/>
     <sheet name="Diploma clocks" sheetId="5" r:id="rId5"/>
@@ -13,8 +13,7 @@
     <sheet name="Inspection self-audit" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Training matrix'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Expiries (automatic)'!$4:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Training matrix'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Supervision tracker'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'DBS re-check log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Diploma clocks'!$4:$4</definedName>
@@ -51,17 +50,17 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9CA3AF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -99,14 +98,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -162,152 +161,150 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="2" max="2" width="95" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Training matrix</t>
+          <t>Start here</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Type each completion date under the course. The Expiries tab does the rest. Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
+          <t>One minute, then you know the whole pack.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Staff member</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Safeguarding Children</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Fire Safety</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Medication Administration</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Food Hygiene</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Health and Safety</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Physical Intervention</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Prevent / Online Safety</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Renews every</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>2 years</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
+          <t>The rule for every tab: type in the plain cells. The coloured cells work themselves out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Training matrix</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Type each person's name, then the date they did each course under "Done on". The cell next to it fills in the expiry and turns green, amber or red on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Supervision tracker</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Name, your cycle in days, date of the last supervision. It flags OVERDUE by itself. Put the manager on the list too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>DBS re-check log</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>For staff on the Update Service: note each status check and it works out when the next one is due.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Diploma clocks</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Start date plus whether they hold the Level 3. The two-year deadline computes itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Governance clocks</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Date each document was last reviewed; next-due dates compute. The monthly visit grid lives here too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Staff file checklist</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>One copy of this tab per person. It is the exact list an inspector reads a file against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Employment gaps</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The most common file failure. Work backwards from their current job; every gap over a month gets one written sentence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Inspection self-audit</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>The eleven things every inspection opens with. Grade yourself honestly.</t>
+        </is>
+      </c>
+    </row>
     <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Each tab has an example row you can overtype or delete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
@@ -319,720 +316,837 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="13" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="13" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Expiry dates, worked out for you</t>
+          <t>Training matrix</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nothing to type here. Red has expired, amber is due within 30 days, green is fine. Check it every Monday.</t>
+          <t>Type the name, then the date each course was done under "Done on". The Expires cell beside it fills in and colours itself: red has run out, amber is due within 30 days, green is fine. Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Staff member</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Safeguarding Children</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Fire Safety</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Medication Administration</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Food Hygiene</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Health and Safety</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Physical Intervention</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Prevent / Online Safety</t>
-        </is>
-      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Safeguarding Children (renews every 1 year)</t>
+        </is>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>First Aid (renews every 3 years)</t>
+        </is>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Fire Safety (renews every 1 year)</t>
+        </is>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Medication Administration (renews every 1 year)</t>
+        </is>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Food Hygiene (renews every 3 years)</t>
+        </is>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Health and Safety (renews every 1 year)</t>
+        </is>
+      </c>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Physical Intervention (renews every 1 year)</t>
+        </is>
+      </c>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>Prevent / Online Safety (renews every 2 years)</t>
+        </is>
+      </c>
+      <c r="Q4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Renews every</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>3 years</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>2 years</t>
+      <c r="A5" s="4"/>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>Done on</t>
+        </is>
+      </c>
+      <c r="Q5" s="6" t="inlineStr">
+        <is>
+          <t>Expires (auto)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6">
-        <f>IF('Training matrix'!A6="","",'Training matrix'!A6)</f>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Example, overtype or delete me</t>
+        </is>
       </c>
       <c r="B6" s="7">
-        <f>IF('Training matrix'!B6="","",EDATE('Training matrix'!B6,12))</f>
+        <v>45859</v>
       </c>
       <c r="C6" s="7">
-        <f>IF('Training matrix'!C6="","",EDATE('Training matrix'!C6,36))</f>
+        <f>IF(B6="","",EDATE(B6,12))</f>
       </c>
       <c r="D6" s="7">
-        <f>IF('Training matrix'!D6="","",EDATE('Training matrix'!D6,12))</f>
+        <v>45259</v>
       </c>
       <c r="E6" s="7">
-        <f>IF('Training matrix'!E6="","",EDATE('Training matrix'!E6,12))</f>
+        <f>IF(D6="","",EDATE(D6,36))</f>
       </c>
       <c r="F6" s="7">
-        <f>IF('Training matrix'!F6="","",EDATE('Training matrix'!F6,36))</f>
+        <v>45909</v>
       </c>
       <c r="G6" s="7">
-        <f>IF('Training matrix'!G6="","",EDATE('Training matrix'!G6,12))</f>
-      </c>
-      <c r="H6" s="7">
-        <f>IF('Training matrix'!H6="","",EDATE('Training matrix'!H6,12))</f>
+        <f>IF(F6="","",EDATE(F6,12))</f>
       </c>
       <c r="I6" s="7">
-        <f>IF('Training matrix'!I6="","",EDATE('Training matrix'!I6,24))</f>
+        <f>IF(H6="","",EDATE(H6,12))</f>
+      </c>
+      <c r="K6" s="7">
+        <f>IF(J6="","",EDATE(J6,36))</f>
+      </c>
+      <c r="M6" s="7">
+        <f>IF(L6="","",EDATE(L6,12))</f>
+      </c>
+      <c r="O6" s="7">
+        <f>IF(N6="","",EDATE(N6,12))</f>
+      </c>
+      <c r="Q6" s="7">
+        <f>IF(P6="","",EDATE(P6,24))</f>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6">
-        <f>IF('Training matrix'!A7="","",'Training matrix'!A7)</f>
-      </c>
-      <c r="B7" s="7">
-        <f>IF('Training matrix'!B7="","",EDATE('Training matrix'!B7,12))</f>
-      </c>
       <c r="C7" s="7">
-        <f>IF('Training matrix'!C7="","",EDATE('Training matrix'!C7,36))</f>
-      </c>
-      <c r="D7" s="7">
-        <f>IF('Training matrix'!D7="","",EDATE('Training matrix'!D7,12))</f>
+        <f>IF(B7="","",EDATE(B7,12))</f>
       </c>
       <c r="E7" s="7">
-        <f>IF('Training matrix'!E7="","",EDATE('Training matrix'!E7,12))</f>
-      </c>
-      <c r="F7" s="7">
-        <f>IF('Training matrix'!F7="","",EDATE('Training matrix'!F7,36))</f>
+        <f>IF(D7="","",EDATE(D7,36))</f>
       </c>
       <c r="G7" s="7">
-        <f>IF('Training matrix'!G7="","",EDATE('Training matrix'!G7,12))</f>
-      </c>
-      <c r="H7" s="7">
-        <f>IF('Training matrix'!H7="","",EDATE('Training matrix'!H7,12))</f>
+        <f>IF(F7="","",EDATE(F7,12))</f>
       </c>
       <c r="I7" s="7">
-        <f>IF('Training matrix'!I7="","",EDATE('Training matrix'!I7,24))</f>
+        <f>IF(H7="","",EDATE(H7,12))</f>
+      </c>
+      <c r="K7" s="7">
+        <f>IF(J7="","",EDATE(J7,36))</f>
+      </c>
+      <c r="M7" s="7">
+        <f>IF(L7="","",EDATE(L7,12))</f>
+      </c>
+      <c r="O7" s="7">
+        <f>IF(N7="","",EDATE(N7,12))</f>
+      </c>
+      <c r="Q7" s="7">
+        <f>IF(P7="","",EDATE(P7,24))</f>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6">
-        <f>IF('Training matrix'!A8="","",'Training matrix'!A8)</f>
-      </c>
-      <c r="B8" s="7">
-        <f>IF('Training matrix'!B8="","",EDATE('Training matrix'!B8,12))</f>
-      </c>
       <c r="C8" s="7">
-        <f>IF('Training matrix'!C8="","",EDATE('Training matrix'!C8,36))</f>
-      </c>
-      <c r="D8" s="7">
-        <f>IF('Training matrix'!D8="","",EDATE('Training matrix'!D8,12))</f>
+        <f>IF(B8="","",EDATE(B8,12))</f>
       </c>
       <c r="E8" s="7">
-        <f>IF('Training matrix'!E8="","",EDATE('Training matrix'!E8,12))</f>
-      </c>
-      <c r="F8" s="7">
-        <f>IF('Training matrix'!F8="","",EDATE('Training matrix'!F8,36))</f>
+        <f>IF(D8="","",EDATE(D8,36))</f>
       </c>
       <c r="G8" s="7">
-        <f>IF('Training matrix'!G8="","",EDATE('Training matrix'!G8,12))</f>
-      </c>
-      <c r="H8" s="7">
-        <f>IF('Training matrix'!H8="","",EDATE('Training matrix'!H8,12))</f>
+        <f>IF(F8="","",EDATE(F8,12))</f>
       </c>
       <c r="I8" s="7">
-        <f>IF('Training matrix'!I8="","",EDATE('Training matrix'!I8,24))</f>
+        <f>IF(H8="","",EDATE(H8,12))</f>
+      </c>
+      <c r="K8" s="7">
+        <f>IF(J8="","",EDATE(J8,36))</f>
+      </c>
+      <c r="M8" s="7">
+        <f>IF(L8="","",EDATE(L8,12))</f>
+      </c>
+      <c r="O8" s="7">
+        <f>IF(N8="","",EDATE(N8,12))</f>
+      </c>
+      <c r="Q8" s="7">
+        <f>IF(P8="","",EDATE(P8,24))</f>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6">
-        <f>IF('Training matrix'!A9="","",'Training matrix'!A9)</f>
-      </c>
-      <c r="B9" s="7">
-        <f>IF('Training matrix'!B9="","",EDATE('Training matrix'!B9,12))</f>
-      </c>
       <c r="C9" s="7">
-        <f>IF('Training matrix'!C9="","",EDATE('Training matrix'!C9,36))</f>
-      </c>
-      <c r="D9" s="7">
-        <f>IF('Training matrix'!D9="","",EDATE('Training matrix'!D9,12))</f>
+        <f>IF(B9="","",EDATE(B9,12))</f>
       </c>
       <c r="E9" s="7">
-        <f>IF('Training matrix'!E9="","",EDATE('Training matrix'!E9,12))</f>
-      </c>
-      <c r="F9" s="7">
-        <f>IF('Training matrix'!F9="","",EDATE('Training matrix'!F9,36))</f>
+        <f>IF(D9="","",EDATE(D9,36))</f>
       </c>
       <c r="G9" s="7">
-        <f>IF('Training matrix'!G9="","",EDATE('Training matrix'!G9,12))</f>
-      </c>
-      <c r="H9" s="7">
-        <f>IF('Training matrix'!H9="","",EDATE('Training matrix'!H9,12))</f>
+        <f>IF(F9="","",EDATE(F9,12))</f>
       </c>
       <c r="I9" s="7">
-        <f>IF('Training matrix'!I9="","",EDATE('Training matrix'!I9,24))</f>
+        <f>IF(H9="","",EDATE(H9,12))</f>
+      </c>
+      <c r="K9" s="7">
+        <f>IF(J9="","",EDATE(J9,36))</f>
+      </c>
+      <c r="M9" s="7">
+        <f>IF(L9="","",EDATE(L9,12))</f>
+      </c>
+      <c r="O9" s="7">
+        <f>IF(N9="","",EDATE(N9,12))</f>
+      </c>
+      <c r="Q9" s="7">
+        <f>IF(P9="","",EDATE(P9,24))</f>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6">
-        <f>IF('Training matrix'!A10="","",'Training matrix'!A10)</f>
-      </c>
-      <c r="B10" s="7">
-        <f>IF('Training matrix'!B10="","",EDATE('Training matrix'!B10,12))</f>
-      </c>
       <c r="C10" s="7">
-        <f>IF('Training matrix'!C10="","",EDATE('Training matrix'!C10,36))</f>
-      </c>
-      <c r="D10" s="7">
-        <f>IF('Training matrix'!D10="","",EDATE('Training matrix'!D10,12))</f>
+        <f>IF(B10="","",EDATE(B10,12))</f>
       </c>
       <c r="E10" s="7">
-        <f>IF('Training matrix'!E10="","",EDATE('Training matrix'!E10,12))</f>
-      </c>
-      <c r="F10" s="7">
-        <f>IF('Training matrix'!F10="","",EDATE('Training matrix'!F10,36))</f>
+        <f>IF(D10="","",EDATE(D10,36))</f>
       </c>
       <c r="G10" s="7">
-        <f>IF('Training matrix'!G10="","",EDATE('Training matrix'!G10,12))</f>
-      </c>
-      <c r="H10" s="7">
-        <f>IF('Training matrix'!H10="","",EDATE('Training matrix'!H10,12))</f>
+        <f>IF(F10="","",EDATE(F10,12))</f>
       </c>
       <c r="I10" s="7">
-        <f>IF('Training matrix'!I10="","",EDATE('Training matrix'!I10,24))</f>
+        <f>IF(H10="","",EDATE(H10,12))</f>
+      </c>
+      <c r="K10" s="7">
+        <f>IF(J10="","",EDATE(J10,36))</f>
+      </c>
+      <c r="M10" s="7">
+        <f>IF(L10="","",EDATE(L10,12))</f>
+      </c>
+      <c r="O10" s="7">
+        <f>IF(N10="","",EDATE(N10,12))</f>
+      </c>
+      <c r="Q10" s="7">
+        <f>IF(P10="","",EDATE(P10,24))</f>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6">
-        <f>IF('Training matrix'!A11="","",'Training matrix'!A11)</f>
-      </c>
-      <c r="B11" s="7">
-        <f>IF('Training matrix'!B11="","",EDATE('Training matrix'!B11,12))</f>
-      </c>
       <c r="C11" s="7">
-        <f>IF('Training matrix'!C11="","",EDATE('Training matrix'!C11,36))</f>
-      </c>
-      <c r="D11" s="7">
-        <f>IF('Training matrix'!D11="","",EDATE('Training matrix'!D11,12))</f>
+        <f>IF(B11="","",EDATE(B11,12))</f>
       </c>
       <c r="E11" s="7">
-        <f>IF('Training matrix'!E11="","",EDATE('Training matrix'!E11,12))</f>
-      </c>
-      <c r="F11" s="7">
-        <f>IF('Training matrix'!F11="","",EDATE('Training matrix'!F11,36))</f>
+        <f>IF(D11="","",EDATE(D11,36))</f>
       </c>
       <c r="G11" s="7">
-        <f>IF('Training matrix'!G11="","",EDATE('Training matrix'!G11,12))</f>
-      </c>
-      <c r="H11" s="7">
-        <f>IF('Training matrix'!H11="","",EDATE('Training matrix'!H11,12))</f>
+        <f>IF(F11="","",EDATE(F11,12))</f>
       </c>
       <c r="I11" s="7">
-        <f>IF('Training matrix'!I11="","",EDATE('Training matrix'!I11,24))</f>
+        <f>IF(H11="","",EDATE(H11,12))</f>
+      </c>
+      <c r="K11" s="7">
+        <f>IF(J11="","",EDATE(J11,36))</f>
+      </c>
+      <c r="M11" s="7">
+        <f>IF(L11="","",EDATE(L11,12))</f>
+      </c>
+      <c r="O11" s="7">
+        <f>IF(N11="","",EDATE(N11,12))</f>
+      </c>
+      <c r="Q11" s="7">
+        <f>IF(P11="","",EDATE(P11,24))</f>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6">
-        <f>IF('Training matrix'!A12="","",'Training matrix'!A12)</f>
-      </c>
-      <c r="B12" s="7">
-        <f>IF('Training matrix'!B12="","",EDATE('Training matrix'!B12,12))</f>
-      </c>
       <c r="C12" s="7">
-        <f>IF('Training matrix'!C12="","",EDATE('Training matrix'!C12,36))</f>
-      </c>
-      <c r="D12" s="7">
-        <f>IF('Training matrix'!D12="","",EDATE('Training matrix'!D12,12))</f>
+        <f>IF(B12="","",EDATE(B12,12))</f>
       </c>
       <c r="E12" s="7">
-        <f>IF('Training matrix'!E12="","",EDATE('Training matrix'!E12,12))</f>
-      </c>
-      <c r="F12" s="7">
-        <f>IF('Training matrix'!F12="","",EDATE('Training matrix'!F12,36))</f>
+        <f>IF(D12="","",EDATE(D12,36))</f>
       </c>
       <c r="G12" s="7">
-        <f>IF('Training matrix'!G12="","",EDATE('Training matrix'!G12,12))</f>
-      </c>
-      <c r="H12" s="7">
-        <f>IF('Training matrix'!H12="","",EDATE('Training matrix'!H12,12))</f>
+        <f>IF(F12="","",EDATE(F12,12))</f>
       </c>
       <c r="I12" s="7">
-        <f>IF('Training matrix'!I12="","",EDATE('Training matrix'!I12,24))</f>
+        <f>IF(H12="","",EDATE(H12,12))</f>
+      </c>
+      <c r="K12" s="7">
+        <f>IF(J12="","",EDATE(J12,36))</f>
+      </c>
+      <c r="M12" s="7">
+        <f>IF(L12="","",EDATE(L12,12))</f>
+      </c>
+      <c r="O12" s="7">
+        <f>IF(N12="","",EDATE(N12,12))</f>
+      </c>
+      <c r="Q12" s="7">
+        <f>IF(P12="","",EDATE(P12,24))</f>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6">
-        <f>IF('Training matrix'!A13="","",'Training matrix'!A13)</f>
-      </c>
-      <c r="B13" s="7">
-        <f>IF('Training matrix'!B13="","",EDATE('Training matrix'!B13,12))</f>
-      </c>
       <c r="C13" s="7">
-        <f>IF('Training matrix'!C13="","",EDATE('Training matrix'!C13,36))</f>
-      </c>
-      <c r="D13" s="7">
-        <f>IF('Training matrix'!D13="","",EDATE('Training matrix'!D13,12))</f>
+        <f>IF(B13="","",EDATE(B13,12))</f>
       </c>
       <c r="E13" s="7">
-        <f>IF('Training matrix'!E13="","",EDATE('Training matrix'!E13,12))</f>
-      </c>
-      <c r="F13" s="7">
-        <f>IF('Training matrix'!F13="","",EDATE('Training matrix'!F13,36))</f>
+        <f>IF(D13="","",EDATE(D13,36))</f>
       </c>
       <c r="G13" s="7">
-        <f>IF('Training matrix'!G13="","",EDATE('Training matrix'!G13,12))</f>
-      </c>
-      <c r="H13" s="7">
-        <f>IF('Training matrix'!H13="","",EDATE('Training matrix'!H13,12))</f>
+        <f>IF(F13="","",EDATE(F13,12))</f>
       </c>
       <c r="I13" s="7">
-        <f>IF('Training matrix'!I13="","",EDATE('Training matrix'!I13,24))</f>
+        <f>IF(H13="","",EDATE(H13,12))</f>
+      </c>
+      <c r="K13" s="7">
+        <f>IF(J13="","",EDATE(J13,36))</f>
+      </c>
+      <c r="M13" s="7">
+        <f>IF(L13="","",EDATE(L13,12))</f>
+      </c>
+      <c r="O13" s="7">
+        <f>IF(N13="","",EDATE(N13,12))</f>
+      </c>
+      <c r="Q13" s="7">
+        <f>IF(P13="","",EDATE(P13,24))</f>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6">
-        <f>IF('Training matrix'!A14="","",'Training matrix'!A14)</f>
-      </c>
-      <c r="B14" s="7">
-        <f>IF('Training matrix'!B14="","",EDATE('Training matrix'!B14,12))</f>
-      </c>
       <c r="C14" s="7">
-        <f>IF('Training matrix'!C14="","",EDATE('Training matrix'!C14,36))</f>
-      </c>
-      <c r="D14" s="7">
-        <f>IF('Training matrix'!D14="","",EDATE('Training matrix'!D14,12))</f>
+        <f>IF(B14="","",EDATE(B14,12))</f>
       </c>
       <c r="E14" s="7">
-        <f>IF('Training matrix'!E14="","",EDATE('Training matrix'!E14,12))</f>
-      </c>
-      <c r="F14" s="7">
-        <f>IF('Training matrix'!F14="","",EDATE('Training matrix'!F14,36))</f>
+        <f>IF(D14="","",EDATE(D14,36))</f>
       </c>
       <c r="G14" s="7">
-        <f>IF('Training matrix'!G14="","",EDATE('Training matrix'!G14,12))</f>
-      </c>
-      <c r="H14" s="7">
-        <f>IF('Training matrix'!H14="","",EDATE('Training matrix'!H14,12))</f>
+        <f>IF(F14="","",EDATE(F14,12))</f>
       </c>
       <c r="I14" s="7">
-        <f>IF('Training matrix'!I14="","",EDATE('Training matrix'!I14,24))</f>
+        <f>IF(H14="","",EDATE(H14,12))</f>
+      </c>
+      <c r="K14" s="7">
+        <f>IF(J14="","",EDATE(J14,36))</f>
+      </c>
+      <c r="M14" s="7">
+        <f>IF(L14="","",EDATE(L14,12))</f>
+      </c>
+      <c r="O14" s="7">
+        <f>IF(N14="","",EDATE(N14,12))</f>
+      </c>
+      <c r="Q14" s="7">
+        <f>IF(P14="","",EDATE(P14,24))</f>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6">
-        <f>IF('Training matrix'!A15="","",'Training matrix'!A15)</f>
-      </c>
-      <c r="B15" s="7">
-        <f>IF('Training matrix'!B15="","",EDATE('Training matrix'!B15,12))</f>
-      </c>
       <c r="C15" s="7">
-        <f>IF('Training matrix'!C15="","",EDATE('Training matrix'!C15,36))</f>
-      </c>
-      <c r="D15" s="7">
-        <f>IF('Training matrix'!D15="","",EDATE('Training matrix'!D15,12))</f>
+        <f>IF(B15="","",EDATE(B15,12))</f>
       </c>
       <c r="E15" s="7">
-        <f>IF('Training matrix'!E15="","",EDATE('Training matrix'!E15,12))</f>
-      </c>
-      <c r="F15" s="7">
-        <f>IF('Training matrix'!F15="","",EDATE('Training matrix'!F15,36))</f>
+        <f>IF(D15="","",EDATE(D15,36))</f>
       </c>
       <c r="G15" s="7">
-        <f>IF('Training matrix'!G15="","",EDATE('Training matrix'!G15,12))</f>
-      </c>
-      <c r="H15" s="7">
-        <f>IF('Training matrix'!H15="","",EDATE('Training matrix'!H15,12))</f>
+        <f>IF(F15="","",EDATE(F15,12))</f>
       </c>
       <c r="I15" s="7">
-        <f>IF('Training matrix'!I15="","",EDATE('Training matrix'!I15,24))</f>
+        <f>IF(H15="","",EDATE(H15,12))</f>
+      </c>
+      <c r="K15" s="7">
+        <f>IF(J15="","",EDATE(J15,36))</f>
+      </c>
+      <c r="M15" s="7">
+        <f>IF(L15="","",EDATE(L15,12))</f>
+      </c>
+      <c r="O15" s="7">
+        <f>IF(N15="","",EDATE(N15,12))</f>
+      </c>
+      <c r="Q15" s="7">
+        <f>IF(P15="","",EDATE(P15,24))</f>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6">
-        <f>IF('Training matrix'!A16="","",'Training matrix'!A16)</f>
-      </c>
-      <c r="B16" s="7">
-        <f>IF('Training matrix'!B16="","",EDATE('Training matrix'!B16,12))</f>
-      </c>
       <c r="C16" s="7">
-        <f>IF('Training matrix'!C16="","",EDATE('Training matrix'!C16,36))</f>
-      </c>
-      <c r="D16" s="7">
-        <f>IF('Training matrix'!D16="","",EDATE('Training matrix'!D16,12))</f>
+        <f>IF(B16="","",EDATE(B16,12))</f>
       </c>
       <c r="E16" s="7">
-        <f>IF('Training matrix'!E16="","",EDATE('Training matrix'!E16,12))</f>
-      </c>
-      <c r="F16" s="7">
-        <f>IF('Training matrix'!F16="","",EDATE('Training matrix'!F16,36))</f>
+        <f>IF(D16="","",EDATE(D16,36))</f>
       </c>
       <c r="G16" s="7">
-        <f>IF('Training matrix'!G16="","",EDATE('Training matrix'!G16,12))</f>
-      </c>
-      <c r="H16" s="7">
-        <f>IF('Training matrix'!H16="","",EDATE('Training matrix'!H16,12))</f>
+        <f>IF(F16="","",EDATE(F16,12))</f>
       </c>
       <c r="I16" s="7">
-        <f>IF('Training matrix'!I16="","",EDATE('Training matrix'!I16,24))</f>
+        <f>IF(H16="","",EDATE(H16,12))</f>
+      </c>
+      <c r="K16" s="7">
+        <f>IF(J16="","",EDATE(J16,36))</f>
+      </c>
+      <c r="M16" s="7">
+        <f>IF(L16="","",EDATE(L16,12))</f>
+      </c>
+      <c r="O16" s="7">
+        <f>IF(N16="","",EDATE(N16,12))</f>
+      </c>
+      <c r="Q16" s="7">
+        <f>IF(P16="","",EDATE(P16,24))</f>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6">
-        <f>IF('Training matrix'!A17="","",'Training matrix'!A17)</f>
-      </c>
-      <c r="B17" s="7">
-        <f>IF('Training matrix'!B17="","",EDATE('Training matrix'!B17,12))</f>
-      </c>
       <c r="C17" s="7">
-        <f>IF('Training matrix'!C17="","",EDATE('Training matrix'!C17,36))</f>
-      </c>
-      <c r="D17" s="7">
-        <f>IF('Training matrix'!D17="","",EDATE('Training matrix'!D17,12))</f>
+        <f>IF(B17="","",EDATE(B17,12))</f>
       </c>
       <c r="E17" s="7">
-        <f>IF('Training matrix'!E17="","",EDATE('Training matrix'!E17,12))</f>
-      </c>
-      <c r="F17" s="7">
-        <f>IF('Training matrix'!F17="","",EDATE('Training matrix'!F17,36))</f>
+        <f>IF(D17="","",EDATE(D17,36))</f>
       </c>
       <c r="G17" s="7">
-        <f>IF('Training matrix'!G17="","",EDATE('Training matrix'!G17,12))</f>
-      </c>
-      <c r="H17" s="7">
-        <f>IF('Training matrix'!H17="","",EDATE('Training matrix'!H17,12))</f>
+        <f>IF(F17="","",EDATE(F17,12))</f>
       </c>
       <c r="I17" s="7">
-        <f>IF('Training matrix'!I17="","",EDATE('Training matrix'!I17,24))</f>
+        <f>IF(H17="","",EDATE(H17,12))</f>
+      </c>
+      <c r="K17" s="7">
+        <f>IF(J17="","",EDATE(J17,36))</f>
+      </c>
+      <c r="M17" s="7">
+        <f>IF(L17="","",EDATE(L17,12))</f>
+      </c>
+      <c r="O17" s="7">
+        <f>IF(N17="","",EDATE(N17,12))</f>
+      </c>
+      <c r="Q17" s="7">
+        <f>IF(P17="","",EDATE(P17,24))</f>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6">
-        <f>IF('Training matrix'!A18="","",'Training matrix'!A18)</f>
-      </c>
-      <c r="B18" s="7">
-        <f>IF('Training matrix'!B18="","",EDATE('Training matrix'!B18,12))</f>
-      </c>
       <c r="C18" s="7">
-        <f>IF('Training matrix'!C18="","",EDATE('Training matrix'!C18,36))</f>
-      </c>
-      <c r="D18" s="7">
-        <f>IF('Training matrix'!D18="","",EDATE('Training matrix'!D18,12))</f>
+        <f>IF(B18="","",EDATE(B18,12))</f>
       </c>
       <c r="E18" s="7">
-        <f>IF('Training matrix'!E18="","",EDATE('Training matrix'!E18,12))</f>
-      </c>
-      <c r="F18" s="7">
-        <f>IF('Training matrix'!F18="","",EDATE('Training matrix'!F18,36))</f>
+        <f>IF(D18="","",EDATE(D18,36))</f>
       </c>
       <c r="G18" s="7">
-        <f>IF('Training matrix'!G18="","",EDATE('Training matrix'!G18,12))</f>
-      </c>
-      <c r="H18" s="7">
-        <f>IF('Training matrix'!H18="","",EDATE('Training matrix'!H18,12))</f>
+        <f>IF(F18="","",EDATE(F18,12))</f>
       </c>
       <c r="I18" s="7">
-        <f>IF('Training matrix'!I18="","",EDATE('Training matrix'!I18,24))</f>
+        <f>IF(H18="","",EDATE(H18,12))</f>
+      </c>
+      <c r="K18" s="7">
+        <f>IF(J18="","",EDATE(J18,36))</f>
+      </c>
+      <c r="M18" s="7">
+        <f>IF(L18="","",EDATE(L18,12))</f>
+      </c>
+      <c r="O18" s="7">
+        <f>IF(N18="","",EDATE(N18,12))</f>
+      </c>
+      <c r="Q18" s="7">
+        <f>IF(P18="","",EDATE(P18,24))</f>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6">
-        <f>IF('Training matrix'!A19="","",'Training matrix'!A19)</f>
-      </c>
-      <c r="B19" s="7">
-        <f>IF('Training matrix'!B19="","",EDATE('Training matrix'!B19,12))</f>
-      </c>
       <c r="C19" s="7">
-        <f>IF('Training matrix'!C19="","",EDATE('Training matrix'!C19,36))</f>
-      </c>
-      <c r="D19" s="7">
-        <f>IF('Training matrix'!D19="","",EDATE('Training matrix'!D19,12))</f>
+        <f>IF(B19="","",EDATE(B19,12))</f>
       </c>
       <c r="E19" s="7">
-        <f>IF('Training matrix'!E19="","",EDATE('Training matrix'!E19,12))</f>
-      </c>
-      <c r="F19" s="7">
-        <f>IF('Training matrix'!F19="","",EDATE('Training matrix'!F19,36))</f>
+        <f>IF(D19="","",EDATE(D19,36))</f>
       </c>
       <c r="G19" s="7">
-        <f>IF('Training matrix'!G19="","",EDATE('Training matrix'!G19,12))</f>
-      </c>
-      <c r="H19" s="7">
-        <f>IF('Training matrix'!H19="","",EDATE('Training matrix'!H19,12))</f>
+        <f>IF(F19="","",EDATE(F19,12))</f>
       </c>
       <c r="I19" s="7">
-        <f>IF('Training matrix'!I19="","",EDATE('Training matrix'!I19,24))</f>
+        <f>IF(H19="","",EDATE(H19,12))</f>
+      </c>
+      <c r="K19" s="7">
+        <f>IF(J19="","",EDATE(J19,36))</f>
+      </c>
+      <c r="M19" s="7">
+        <f>IF(L19="","",EDATE(L19,12))</f>
+      </c>
+      <c r="O19" s="7">
+        <f>IF(N19="","",EDATE(N19,12))</f>
+      </c>
+      <c r="Q19" s="7">
+        <f>IF(P19="","",EDATE(P19,24))</f>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6">
-        <f>IF('Training matrix'!A20="","",'Training matrix'!A20)</f>
-      </c>
-      <c r="B20" s="7">
-        <f>IF('Training matrix'!B20="","",EDATE('Training matrix'!B20,12))</f>
-      </c>
       <c r="C20" s="7">
-        <f>IF('Training matrix'!C20="","",EDATE('Training matrix'!C20,36))</f>
-      </c>
-      <c r="D20" s="7">
-        <f>IF('Training matrix'!D20="","",EDATE('Training matrix'!D20,12))</f>
+        <f>IF(B20="","",EDATE(B20,12))</f>
       </c>
       <c r="E20" s="7">
-        <f>IF('Training matrix'!E20="","",EDATE('Training matrix'!E20,12))</f>
-      </c>
-      <c r="F20" s="7">
-        <f>IF('Training matrix'!F20="","",EDATE('Training matrix'!F20,36))</f>
+        <f>IF(D20="","",EDATE(D20,36))</f>
       </c>
       <c r="G20" s="7">
-        <f>IF('Training matrix'!G20="","",EDATE('Training matrix'!G20,12))</f>
-      </c>
-      <c r="H20" s="7">
-        <f>IF('Training matrix'!H20="","",EDATE('Training matrix'!H20,12))</f>
+        <f>IF(F20="","",EDATE(F20,12))</f>
       </c>
       <c r="I20" s="7">
-        <f>IF('Training matrix'!I20="","",EDATE('Training matrix'!I20,24))</f>
+        <f>IF(H20="","",EDATE(H20,12))</f>
+      </c>
+      <c r="K20" s="7">
+        <f>IF(J20="","",EDATE(J20,36))</f>
+      </c>
+      <c r="M20" s="7">
+        <f>IF(L20="","",EDATE(L20,12))</f>
+      </c>
+      <c r="O20" s="7">
+        <f>IF(N20="","",EDATE(N20,12))</f>
+      </c>
+      <c r="Q20" s="7">
+        <f>IF(P20="","",EDATE(P20,24))</f>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6">
-        <f>IF('Training matrix'!A21="","",'Training matrix'!A21)</f>
-      </c>
-      <c r="B21" s="7">
-        <f>IF('Training matrix'!B21="","",EDATE('Training matrix'!B21,12))</f>
-      </c>
       <c r="C21" s="7">
-        <f>IF('Training matrix'!C21="","",EDATE('Training matrix'!C21,36))</f>
-      </c>
-      <c r="D21" s="7">
-        <f>IF('Training matrix'!D21="","",EDATE('Training matrix'!D21,12))</f>
+        <f>IF(B21="","",EDATE(B21,12))</f>
       </c>
       <c r="E21" s="7">
-        <f>IF('Training matrix'!E21="","",EDATE('Training matrix'!E21,12))</f>
-      </c>
-      <c r="F21" s="7">
-        <f>IF('Training matrix'!F21="","",EDATE('Training matrix'!F21,36))</f>
+        <f>IF(D21="","",EDATE(D21,36))</f>
       </c>
       <c r="G21" s="7">
-        <f>IF('Training matrix'!G21="","",EDATE('Training matrix'!G21,12))</f>
-      </c>
-      <c r="H21" s="7">
-        <f>IF('Training matrix'!H21="","",EDATE('Training matrix'!H21,12))</f>
+        <f>IF(F21="","",EDATE(F21,12))</f>
       </c>
       <c r="I21" s="7">
-        <f>IF('Training matrix'!I21="","",EDATE('Training matrix'!I21,24))</f>
+        <f>IF(H21="","",EDATE(H21,12))</f>
+      </c>
+      <c r="K21" s="7">
+        <f>IF(J21="","",EDATE(J21,36))</f>
+      </c>
+      <c r="M21" s="7">
+        <f>IF(L21="","",EDATE(L21,12))</f>
+      </c>
+      <c r="O21" s="7">
+        <f>IF(N21="","",EDATE(N21,12))</f>
+      </c>
+      <c r="Q21" s="7">
+        <f>IF(P21="","",EDATE(P21,24))</f>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6">
-        <f>IF('Training matrix'!A22="","",'Training matrix'!A22)</f>
-      </c>
-      <c r="B22" s="7">
-        <f>IF('Training matrix'!B22="","",EDATE('Training matrix'!B22,12))</f>
-      </c>
       <c r="C22" s="7">
-        <f>IF('Training matrix'!C22="","",EDATE('Training matrix'!C22,36))</f>
-      </c>
-      <c r="D22" s="7">
-        <f>IF('Training matrix'!D22="","",EDATE('Training matrix'!D22,12))</f>
+        <f>IF(B22="","",EDATE(B22,12))</f>
       </c>
       <c r="E22" s="7">
-        <f>IF('Training matrix'!E22="","",EDATE('Training matrix'!E22,12))</f>
-      </c>
-      <c r="F22" s="7">
-        <f>IF('Training matrix'!F22="","",EDATE('Training matrix'!F22,36))</f>
+        <f>IF(D22="","",EDATE(D22,36))</f>
       </c>
       <c r="G22" s="7">
-        <f>IF('Training matrix'!G22="","",EDATE('Training matrix'!G22,12))</f>
-      </c>
-      <c r="H22" s="7">
-        <f>IF('Training matrix'!H22="","",EDATE('Training matrix'!H22,12))</f>
+        <f>IF(F22="","",EDATE(F22,12))</f>
       </c>
       <c r="I22" s="7">
-        <f>IF('Training matrix'!I22="","",EDATE('Training matrix'!I22,24))</f>
+        <f>IF(H22="","",EDATE(H22,12))</f>
+      </c>
+      <c r="K22" s="7">
+        <f>IF(J22="","",EDATE(J22,36))</f>
+      </c>
+      <c r="M22" s="7">
+        <f>IF(L22="","",EDATE(L22,12))</f>
+      </c>
+      <c r="O22" s="7">
+        <f>IF(N22="","",EDATE(N22,12))</f>
+      </c>
+      <c r="Q22" s="7">
+        <f>IF(P22="","",EDATE(P22,24))</f>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6">
-        <f>IF('Training matrix'!A23="","",'Training matrix'!A23)</f>
-      </c>
-      <c r="B23" s="7">
-        <f>IF('Training matrix'!B23="","",EDATE('Training matrix'!B23,12))</f>
-      </c>
       <c r="C23" s="7">
-        <f>IF('Training matrix'!C23="","",EDATE('Training matrix'!C23,36))</f>
-      </c>
-      <c r="D23" s="7">
-        <f>IF('Training matrix'!D23="","",EDATE('Training matrix'!D23,12))</f>
+        <f>IF(B23="","",EDATE(B23,12))</f>
       </c>
       <c r="E23" s="7">
-        <f>IF('Training matrix'!E23="","",EDATE('Training matrix'!E23,12))</f>
-      </c>
-      <c r="F23" s="7">
-        <f>IF('Training matrix'!F23="","",EDATE('Training matrix'!F23,36))</f>
+        <f>IF(D23="","",EDATE(D23,36))</f>
       </c>
       <c r="G23" s="7">
-        <f>IF('Training matrix'!G23="","",EDATE('Training matrix'!G23,12))</f>
-      </c>
-      <c r="H23" s="7">
-        <f>IF('Training matrix'!H23="","",EDATE('Training matrix'!H23,12))</f>
+        <f>IF(F23="","",EDATE(F23,12))</f>
       </c>
       <c r="I23" s="7">
-        <f>IF('Training matrix'!I23="","",EDATE('Training matrix'!I23,24))</f>
+        <f>IF(H23="","",EDATE(H23,12))</f>
+      </c>
+      <c r="K23" s="7">
+        <f>IF(J23="","",EDATE(J23,36))</f>
+      </c>
+      <c r="M23" s="7">
+        <f>IF(L23="","",EDATE(L23,12))</f>
+      </c>
+      <c r="O23" s="7">
+        <f>IF(N23="","",EDATE(N23,12))</f>
+      </c>
+      <c r="Q23" s="7">
+        <f>IF(P23="","",EDATE(P23,24))</f>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6">
-        <f>IF('Training matrix'!A24="","",'Training matrix'!A24)</f>
-      </c>
-      <c r="B24" s="7">
-        <f>IF('Training matrix'!B24="","",EDATE('Training matrix'!B24,12))</f>
-      </c>
       <c r="C24" s="7">
-        <f>IF('Training matrix'!C24="","",EDATE('Training matrix'!C24,36))</f>
-      </c>
-      <c r="D24" s="7">
-        <f>IF('Training matrix'!D24="","",EDATE('Training matrix'!D24,12))</f>
+        <f>IF(B24="","",EDATE(B24,12))</f>
       </c>
       <c r="E24" s="7">
-        <f>IF('Training matrix'!E24="","",EDATE('Training matrix'!E24,12))</f>
-      </c>
-      <c r="F24" s="7">
-        <f>IF('Training matrix'!F24="","",EDATE('Training matrix'!F24,36))</f>
+        <f>IF(D24="","",EDATE(D24,36))</f>
       </c>
       <c r="G24" s="7">
-        <f>IF('Training matrix'!G24="","",EDATE('Training matrix'!G24,12))</f>
-      </c>
-      <c r="H24" s="7">
-        <f>IF('Training matrix'!H24="","",EDATE('Training matrix'!H24,12))</f>
+        <f>IF(F24="","",EDATE(F24,12))</f>
       </c>
       <c r="I24" s="7">
-        <f>IF('Training matrix'!I24="","",EDATE('Training matrix'!I24,24))</f>
+        <f>IF(H24="","",EDATE(H24,12))</f>
+      </c>
+      <c r="K24" s="7">
+        <f>IF(J24="","",EDATE(J24,36))</f>
+      </c>
+      <c r="M24" s="7">
+        <f>IF(L24="","",EDATE(L24,12))</f>
+      </c>
+      <c r="O24" s="7">
+        <f>IF(N24="","",EDATE(N24,12))</f>
+      </c>
+      <c r="Q24" s="7">
+        <f>IF(P24="","",EDATE(P24,24))</f>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6">
-        <f>IF('Training matrix'!A25="","",'Training matrix'!A25)</f>
-      </c>
-      <c r="B25" s="7">
-        <f>IF('Training matrix'!B25="","",EDATE('Training matrix'!B25,12))</f>
-      </c>
       <c r="C25" s="7">
-        <f>IF('Training matrix'!C25="","",EDATE('Training matrix'!C25,36))</f>
-      </c>
-      <c r="D25" s="7">
-        <f>IF('Training matrix'!D25="","",EDATE('Training matrix'!D25,12))</f>
+        <f>IF(B25="","",EDATE(B25,12))</f>
       </c>
       <c r="E25" s="7">
-        <f>IF('Training matrix'!E25="","",EDATE('Training matrix'!E25,12))</f>
-      </c>
-      <c r="F25" s="7">
-        <f>IF('Training matrix'!F25="","",EDATE('Training matrix'!F25,36))</f>
+        <f>IF(D25="","",EDATE(D25,36))</f>
       </c>
       <c r="G25" s="7">
-        <f>IF('Training matrix'!G25="","",EDATE('Training matrix'!G25,12))</f>
-      </c>
-      <c r="H25" s="7">
-        <f>IF('Training matrix'!H25="","",EDATE('Training matrix'!H25,12))</f>
+        <f>IF(F25="","",EDATE(F25,12))</f>
       </c>
       <c r="I25" s="7">
-        <f>IF('Training matrix'!I25="","",EDATE('Training matrix'!I25,24))</f>
+        <f>IF(H25="","",EDATE(H25,12))</f>
+      </c>
+      <c r="K25" s="7">
+        <f>IF(J25="","",EDATE(J25,36))</f>
+      </c>
+      <c r="M25" s="7">
+        <f>IF(L25="","",EDATE(L25,12))</f>
+      </c>
+      <c r="O25" s="7">
+        <f>IF(N25="","",EDATE(N25,12))</f>
+      </c>
+      <c r="Q25" s="7">
+        <f>IF(P25="","",EDATE(P25,24))</f>
+      </c>
+    </row>
+    <row r="26">
+      <c r="C26" s="7">
+        <f>IF(B26="","",EDATE(B26,12))</f>
+      </c>
+      <c r="E26" s="7">
+        <f>IF(D26="","",EDATE(D26,36))</f>
+      </c>
+      <c r="G26" s="7">
+        <f>IF(F26="","",EDATE(F26,12))</f>
+      </c>
+      <c r="I26" s="7">
+        <f>IF(H26="","",EDATE(H26,12))</f>
+      </c>
+      <c r="K26" s="7">
+        <f>IF(J26="","",EDATE(J26,36))</f>
+      </c>
+      <c r="M26" s="7">
+        <f>IF(L26="","",EDATE(L26,12))</f>
+      </c>
+      <c r="O26" s="7">
+        <f>IF(N26="","",EDATE(N26,12))</f>
+      </c>
+      <c r="Q26" s="7">
+        <f>IF(P26="","",EDATE(P26,24))</f>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="10">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:Q4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B6:I25">
+  <conditionalFormatting sqref="C6:C26">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND(B6&lt;&gt;"",B6&lt;TODAY())</formula>
+      <formula>AND(C6&lt;&gt;"",C6&lt;TODAY())</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>AND(B6&lt;&gt;"",B6&lt;TODAY()+30)</formula>
+      <formula>AND(C6&lt;&gt;"",C6&lt;TODAY()+30)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
-      <formula>AND(B6&lt;&gt;"",B6&gt;=TODAY()+30)</formula>
+      <formula>AND(C6&lt;&gt;"",C6&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6:E26">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>AND(E6&lt;&gt;"",E6&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="5">
+      <formula>AND(E6&lt;&gt;"",E6&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="6">
+      <formula>AND(E6&lt;&gt;"",E6&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6:G26">
+    <cfRule type="expression" dxfId="0" priority="7">
+      <formula>AND(G6&lt;&gt;"",G6&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="8">
+      <formula>AND(G6&lt;&gt;"",G6&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="9">
+      <formula>AND(G6&lt;&gt;"",G6&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:I26">
+    <cfRule type="expression" dxfId="0" priority="10">
+      <formula>AND(I6&lt;&gt;"",I6&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="11">
+      <formula>AND(I6&lt;&gt;"",I6&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="12">
+      <formula>AND(I6&lt;&gt;"",I6&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6:K26">
+    <cfRule type="expression" dxfId="0" priority="13">
+      <formula>AND(K6&lt;&gt;"",K6&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="14">
+      <formula>AND(K6&lt;&gt;"",K6&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="15">
+      <formula>AND(K6&lt;&gt;"",K6&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M6:M26">
+    <cfRule type="expression" dxfId="0" priority="16">
+      <formula>AND(M6&lt;&gt;"",M6&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="17">
+      <formula>AND(M6&lt;&gt;"",M6&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="18">
+      <formula>AND(M6&lt;&gt;"",M6&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O6:O26">
+    <cfRule type="expression" dxfId="0" priority="19">
+      <formula>AND(O6&lt;&gt;"",O6&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="20">
+      <formula>AND(O6&lt;&gt;"",O6&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="21">
+      <formula>AND(O6&lt;&gt;"",O6&gt;=TODAY()+30)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q6:Q26">
+    <cfRule type="expression" dxfId="0" priority="22">
+      <formula>AND(Q6&lt;&gt;"",Q6&lt;TODAY())</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="23">
+      <formula>AND(Q6&lt;&gt;"",Q6&lt;TODAY()+30)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="24">
+      <formula>AND(Q6&lt;&gt;"",Q6&gt;=TODAY()+30)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -1071,34 +1185,34 @@
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Staff member</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Cycle (days)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Last supervision</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Days since</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Example: change or delete this row</t>
         </is>
@@ -1389,39 +1503,39 @@
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Staff member</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Certificate number</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>On the Update Service?</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Last status check</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Next check due</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Example: change or delete this row</t>
         </is>
@@ -1599,29 +1713,29 @@
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Staff member</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Start date</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Holds Level 3? (Yes/No)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Level 3 due by</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Example: change or delete this row</t>
         </is>
@@ -1809,22 +1923,22 @@
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Document</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Last reviewed</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Review every (months)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Next due</t>
         </is>
@@ -1936,29 +2050,29 @@
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>The two visit clocks</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Reg 44 visit date</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Report received</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Actions all closed?</t>
         </is>
@@ -2050,7 +2164,7 @@
     </row>
     <row r="28"/>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Reg 45 quality of care review: due every six months, sent to Ofsted within 28 days of completing it.</t>
         </is>
@@ -2108,27 +2222,27 @@
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>What the file must hold</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>What satisfies it</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>In the file?</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Date checked</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2311,32 +2425,32 @@
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>From (month/year)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>To (month/year)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Employer, course, or what the gap was</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Reason for leaving</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Checked?</t>
         </is>
@@ -2446,22 +2560,22 @@
     </row>
     <row r="3"/>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>The inspector asks for</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Where yours lives today</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Ready / Question / Gap</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>What would make it Ready</t>
         </is>
@@ -2561,7 +2675,7 @@
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
         </is>

</xml_diff>

<commit_message>
Pack workbook v3: Start-here merges, audited formatting
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pack/staffbook-staff-file-pack.xlsx
+++ b/pack/staffbook-staff-file-pack.xlsx
@@ -78,11 +78,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4F7F3"/>
+        <fgColor rgb="FFEFF4EE"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -90,29 +90,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD5D2C4"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD5D2C4"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD5D2C4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD5D2C4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -161,7 +183,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="95" customWidth="1"/>
+    <col min="2" max="2" width="100" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -182,7 +204,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>The rule for every tab: type in the plain cells. The coloured cells work themselves out.</t>
+          <t>The rule for every tab: white cells are yours to type in. Tinted cells work themselves out.</t>
         </is>
       </c>
     </row>
@@ -193,9 +215,9 @@
           <t>Training matrix</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Type each person's name, then the date they did each course under "Done on". The cell next to it fills in the expiry and turns green, amber or red on its own.</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Type each person's name, then the date they did each course under "Done on". The tinted cell beside it fills in the expiry. In Excel and Google Sheets it also turns green, amber or red.</t>
         </is>
       </c>
     </row>
@@ -205,7 +227,7 @@
           <t>Supervision tracker</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Name, your cycle in days, date of the last supervision. It flags OVERDUE by itself. Put the manager on the list too.</t>
         </is>
@@ -217,7 +239,7 @@
           <t>DBS re-check log</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>For staff on the Update Service: note each status check and it works out when the next one is due.</t>
         </is>
@@ -229,7 +251,7 @@
           <t>Diploma clocks</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Start date plus whether they hold the Level 3. The two-year deadline computes itself.</t>
         </is>
@@ -241,7 +263,7 @@
           <t>Governance clocks</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Date each document was last reviewed; next-due dates compute. The monthly visit grid lives here too.</t>
         </is>
@@ -253,7 +275,7 @@
           <t>Staff file checklist</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>One copy of this tab per person. It is the exact list an inspector reads a file against.</t>
         </is>
@@ -265,7 +287,7 @@
           <t>Employment gaps</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>The most common file failure. Work backwards from their current job; every gap over a month gets one written sentence.</t>
         </is>
@@ -277,7 +299,7 @@
           <t>Inspection self-audit</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>The eleven things every inspection opens with. Grade yourself honestly.</t>
         </is>
@@ -285,23 +307,26 @@
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Each tab has an example row you can overtype or delete.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
@@ -345,12 +370,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Type the name, then the date each course was done under "Done on". The Expires cell beside it fills in and colours itself: red has run out, amber is due within 30 days, green is fine. Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
+          <t>Type the name, then the date each course was done under "Done on". The tinted Expires cell beside it fills in by itself. Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Staff member</t>
@@ -407,644 +432,829 @@
     </row>
     <row r="5">
       <c r="A5" s="4"/>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="N5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="O5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
-      <c r="P5" s="6" t="inlineStr">
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>Done on</t>
         </is>
       </c>
-      <c r="Q5" s="6" t="inlineStr">
+      <c r="Q5" s="7" t="inlineStr">
         <is>
           <t>Expires (auto)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Example, overtype or delete me</t>
         </is>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>45859</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="10">
         <f>IF(B6="","",EDATE(B6,12))</f>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="9">
         <v>45259</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="10">
         <f>IF(D6="","",EDATE(D6,36))</f>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="9">
         <v>45909</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="10">
         <f>IF(F6="","",EDATE(F6,12))</f>
       </c>
-      <c r="I6" s="7">
+      <c r="H6" s="11"/>
+      <c r="I6" s="10">
         <f>IF(H6="","",EDATE(H6,12))</f>
       </c>
-      <c r="K6" s="7">
+      <c r="J6" s="11"/>
+      <c r="K6" s="10">
         <f>IF(J6="","",EDATE(J6,36))</f>
       </c>
-      <c r="M6" s="7">
+      <c r="L6" s="11"/>
+      <c r="M6" s="10">
         <f>IF(L6="","",EDATE(L6,12))</f>
       </c>
-      <c r="O6" s="7">
+      <c r="N6" s="11"/>
+      <c r="O6" s="10">
         <f>IF(N6="","",EDATE(N6,12))</f>
       </c>
-      <c r="Q6" s="7">
+      <c r="P6" s="11"/>
+      <c r="Q6" s="10">
         <f>IF(P6="","",EDATE(P6,24))</f>
       </c>
     </row>
     <row r="7">
-      <c r="C7" s="7">
+      <c r="A7" s="5"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="10">
         <f>IF(B7="","",EDATE(B7,12))</f>
       </c>
-      <c r="E7" s="7">
+      <c r="D7" s="11"/>
+      <c r="E7" s="10">
         <f>IF(D7="","",EDATE(D7,36))</f>
       </c>
-      <c r="G7" s="7">
+      <c r="F7" s="11"/>
+      <c r="G7" s="10">
         <f>IF(F7="","",EDATE(F7,12))</f>
       </c>
-      <c r="I7" s="7">
+      <c r="H7" s="11"/>
+      <c r="I7" s="10">
         <f>IF(H7="","",EDATE(H7,12))</f>
       </c>
-      <c r="K7" s="7">
+      <c r="J7" s="11"/>
+      <c r="K7" s="10">
         <f>IF(J7="","",EDATE(J7,36))</f>
       </c>
-      <c r="M7" s="7">
+      <c r="L7" s="11"/>
+      <c r="M7" s="10">
         <f>IF(L7="","",EDATE(L7,12))</f>
       </c>
-      <c r="O7" s="7">
+      <c r="N7" s="11"/>
+      <c r="O7" s="10">
         <f>IF(N7="","",EDATE(N7,12))</f>
       </c>
-      <c r="Q7" s="7">
+      <c r="P7" s="11"/>
+      <c r="Q7" s="10">
         <f>IF(P7="","",EDATE(P7,24))</f>
       </c>
     </row>
     <row r="8">
-      <c r="C8" s="7">
+      <c r="A8" s="5"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="10">
         <f>IF(B8="","",EDATE(B8,12))</f>
       </c>
-      <c r="E8" s="7">
+      <c r="D8" s="11"/>
+      <c r="E8" s="10">
         <f>IF(D8="","",EDATE(D8,36))</f>
       </c>
-      <c r="G8" s="7">
+      <c r="F8" s="11"/>
+      <c r="G8" s="10">
         <f>IF(F8="","",EDATE(F8,12))</f>
       </c>
-      <c r="I8" s="7">
+      <c r="H8" s="11"/>
+      <c r="I8" s="10">
         <f>IF(H8="","",EDATE(H8,12))</f>
       </c>
-      <c r="K8" s="7">
+      <c r="J8" s="11"/>
+      <c r="K8" s="10">
         <f>IF(J8="","",EDATE(J8,36))</f>
       </c>
-      <c r="M8" s="7">
+      <c r="L8" s="11"/>
+      <c r="M8" s="10">
         <f>IF(L8="","",EDATE(L8,12))</f>
       </c>
-      <c r="O8" s="7">
+      <c r="N8" s="11"/>
+      <c r="O8" s="10">
         <f>IF(N8="","",EDATE(N8,12))</f>
       </c>
-      <c r="Q8" s="7">
+      <c r="P8" s="11"/>
+      <c r="Q8" s="10">
         <f>IF(P8="","",EDATE(P8,24))</f>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="7">
+      <c r="A9" s="5"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="10">
         <f>IF(B9="","",EDATE(B9,12))</f>
       </c>
-      <c r="E9" s="7">
+      <c r="D9" s="11"/>
+      <c r="E9" s="10">
         <f>IF(D9="","",EDATE(D9,36))</f>
       </c>
-      <c r="G9" s="7">
+      <c r="F9" s="11"/>
+      <c r="G9" s="10">
         <f>IF(F9="","",EDATE(F9,12))</f>
       </c>
-      <c r="I9" s="7">
+      <c r="H9" s="11"/>
+      <c r="I9" s="10">
         <f>IF(H9="","",EDATE(H9,12))</f>
       </c>
-      <c r="K9" s="7">
+      <c r="J9" s="11"/>
+      <c r="K9" s="10">
         <f>IF(J9="","",EDATE(J9,36))</f>
       </c>
-      <c r="M9" s="7">
+      <c r="L9" s="11"/>
+      <c r="M9" s="10">
         <f>IF(L9="","",EDATE(L9,12))</f>
       </c>
-      <c r="O9" s="7">
+      <c r="N9" s="11"/>
+      <c r="O9" s="10">
         <f>IF(N9="","",EDATE(N9,12))</f>
       </c>
-      <c r="Q9" s="7">
+      <c r="P9" s="11"/>
+      <c r="Q9" s="10">
         <f>IF(P9="","",EDATE(P9,24))</f>
       </c>
     </row>
     <row r="10">
-      <c r="C10" s="7">
+      <c r="A10" s="5"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="10">
         <f>IF(B10="","",EDATE(B10,12))</f>
       </c>
-      <c r="E10" s="7">
+      <c r="D10" s="11"/>
+      <c r="E10" s="10">
         <f>IF(D10="","",EDATE(D10,36))</f>
       </c>
-      <c r="G10" s="7">
+      <c r="F10" s="11"/>
+      <c r="G10" s="10">
         <f>IF(F10="","",EDATE(F10,12))</f>
       </c>
-      <c r="I10" s="7">
+      <c r="H10" s="11"/>
+      <c r="I10" s="10">
         <f>IF(H10="","",EDATE(H10,12))</f>
       </c>
-      <c r="K10" s="7">
+      <c r="J10" s="11"/>
+      <c r="K10" s="10">
         <f>IF(J10="","",EDATE(J10,36))</f>
       </c>
-      <c r="M10" s="7">
+      <c r="L10" s="11"/>
+      <c r="M10" s="10">
         <f>IF(L10="","",EDATE(L10,12))</f>
       </c>
-      <c r="O10" s="7">
+      <c r="N10" s="11"/>
+      <c r="O10" s="10">
         <f>IF(N10="","",EDATE(N10,12))</f>
       </c>
-      <c r="Q10" s="7">
+      <c r="P10" s="11"/>
+      <c r="Q10" s="10">
         <f>IF(P10="","",EDATE(P10,24))</f>
       </c>
     </row>
     <row r="11">
-      <c r="C11" s="7">
+      <c r="A11" s="5"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="10">
         <f>IF(B11="","",EDATE(B11,12))</f>
       </c>
-      <c r="E11" s="7">
+      <c r="D11" s="11"/>
+      <c r="E11" s="10">
         <f>IF(D11="","",EDATE(D11,36))</f>
       </c>
-      <c r="G11" s="7">
+      <c r="F11" s="11"/>
+      <c r="G11" s="10">
         <f>IF(F11="","",EDATE(F11,12))</f>
       </c>
-      <c r="I11" s="7">
+      <c r="H11" s="11"/>
+      <c r="I11" s="10">
         <f>IF(H11="","",EDATE(H11,12))</f>
       </c>
-      <c r="K11" s="7">
+      <c r="J11" s="11"/>
+      <c r="K11" s="10">
         <f>IF(J11="","",EDATE(J11,36))</f>
       </c>
-      <c r="M11" s="7">
+      <c r="L11" s="11"/>
+      <c r="M11" s="10">
         <f>IF(L11="","",EDATE(L11,12))</f>
       </c>
-      <c r="O11" s="7">
+      <c r="N11" s="11"/>
+      <c r="O11" s="10">
         <f>IF(N11="","",EDATE(N11,12))</f>
       </c>
-      <c r="Q11" s="7">
+      <c r="P11" s="11"/>
+      <c r="Q11" s="10">
         <f>IF(P11="","",EDATE(P11,24))</f>
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="7">
+      <c r="A12" s="5"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="10">
         <f>IF(B12="","",EDATE(B12,12))</f>
       </c>
-      <c r="E12" s="7">
+      <c r="D12" s="11"/>
+      <c r="E12" s="10">
         <f>IF(D12="","",EDATE(D12,36))</f>
       </c>
-      <c r="G12" s="7">
+      <c r="F12" s="11"/>
+      <c r="G12" s="10">
         <f>IF(F12="","",EDATE(F12,12))</f>
       </c>
-      <c r="I12" s="7">
+      <c r="H12" s="11"/>
+      <c r="I12" s="10">
         <f>IF(H12="","",EDATE(H12,12))</f>
       </c>
-      <c r="K12" s="7">
+      <c r="J12" s="11"/>
+      <c r="K12" s="10">
         <f>IF(J12="","",EDATE(J12,36))</f>
       </c>
-      <c r="M12" s="7">
+      <c r="L12" s="11"/>
+      <c r="M12" s="10">
         <f>IF(L12="","",EDATE(L12,12))</f>
       </c>
-      <c r="O12" s="7">
+      <c r="N12" s="11"/>
+      <c r="O12" s="10">
         <f>IF(N12="","",EDATE(N12,12))</f>
       </c>
-      <c r="Q12" s="7">
+      <c r="P12" s="11"/>
+      <c r="Q12" s="10">
         <f>IF(P12="","",EDATE(P12,24))</f>
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="7">
+      <c r="A13" s="5"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="10">
         <f>IF(B13="","",EDATE(B13,12))</f>
       </c>
-      <c r="E13" s="7">
+      <c r="D13" s="11"/>
+      <c r="E13" s="10">
         <f>IF(D13="","",EDATE(D13,36))</f>
       </c>
-      <c r="G13" s="7">
+      <c r="F13" s="11"/>
+      <c r="G13" s="10">
         <f>IF(F13="","",EDATE(F13,12))</f>
       </c>
-      <c r="I13" s="7">
+      <c r="H13" s="11"/>
+      <c r="I13" s="10">
         <f>IF(H13="","",EDATE(H13,12))</f>
       </c>
-      <c r="K13" s="7">
+      <c r="J13" s="11"/>
+      <c r="K13" s="10">
         <f>IF(J13="","",EDATE(J13,36))</f>
       </c>
-      <c r="M13" s="7">
+      <c r="L13" s="11"/>
+      <c r="M13" s="10">
         <f>IF(L13="","",EDATE(L13,12))</f>
       </c>
-      <c r="O13" s="7">
+      <c r="N13" s="11"/>
+      <c r="O13" s="10">
         <f>IF(N13="","",EDATE(N13,12))</f>
       </c>
-      <c r="Q13" s="7">
+      <c r="P13" s="11"/>
+      <c r="Q13" s="10">
         <f>IF(P13="","",EDATE(P13,24))</f>
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="7">
+      <c r="A14" s="5"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="10">
         <f>IF(B14="","",EDATE(B14,12))</f>
       </c>
-      <c r="E14" s="7">
+      <c r="D14" s="11"/>
+      <c r="E14" s="10">
         <f>IF(D14="","",EDATE(D14,36))</f>
       </c>
-      <c r="G14" s="7">
+      <c r="F14" s="11"/>
+      <c r="G14" s="10">
         <f>IF(F14="","",EDATE(F14,12))</f>
       </c>
-      <c r="I14" s="7">
+      <c r="H14" s="11"/>
+      <c r="I14" s="10">
         <f>IF(H14="","",EDATE(H14,12))</f>
       </c>
-      <c r="K14" s="7">
+      <c r="J14" s="11"/>
+      <c r="K14" s="10">
         <f>IF(J14="","",EDATE(J14,36))</f>
       </c>
-      <c r="M14" s="7">
+      <c r="L14" s="11"/>
+      <c r="M14" s="10">
         <f>IF(L14="","",EDATE(L14,12))</f>
       </c>
-      <c r="O14" s="7">
+      <c r="N14" s="11"/>
+      <c r="O14" s="10">
         <f>IF(N14="","",EDATE(N14,12))</f>
       </c>
-      <c r="Q14" s="7">
+      <c r="P14" s="11"/>
+      <c r="Q14" s="10">
         <f>IF(P14="","",EDATE(P14,24))</f>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="7">
+      <c r="A15" s="5"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="10">
         <f>IF(B15="","",EDATE(B15,12))</f>
       </c>
-      <c r="E15" s="7">
+      <c r="D15" s="11"/>
+      <c r="E15" s="10">
         <f>IF(D15="","",EDATE(D15,36))</f>
       </c>
-      <c r="G15" s="7">
+      <c r="F15" s="11"/>
+      <c r="G15" s="10">
         <f>IF(F15="","",EDATE(F15,12))</f>
       </c>
-      <c r="I15" s="7">
+      <c r="H15" s="11"/>
+      <c r="I15" s="10">
         <f>IF(H15="","",EDATE(H15,12))</f>
       </c>
-      <c r="K15" s="7">
+      <c r="J15" s="11"/>
+      <c r="K15" s="10">
         <f>IF(J15="","",EDATE(J15,36))</f>
       </c>
-      <c r="M15" s="7">
+      <c r="L15" s="11"/>
+      <c r="M15" s="10">
         <f>IF(L15="","",EDATE(L15,12))</f>
       </c>
-      <c r="O15" s="7">
+      <c r="N15" s="11"/>
+      <c r="O15" s="10">
         <f>IF(N15="","",EDATE(N15,12))</f>
       </c>
-      <c r="Q15" s="7">
+      <c r="P15" s="11"/>
+      <c r="Q15" s="10">
         <f>IF(P15="","",EDATE(P15,24))</f>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="7">
+      <c r="A16" s="5"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="10">
         <f>IF(B16="","",EDATE(B16,12))</f>
       </c>
-      <c r="E16" s="7">
+      <c r="D16" s="11"/>
+      <c r="E16" s="10">
         <f>IF(D16="","",EDATE(D16,36))</f>
       </c>
-      <c r="G16" s="7">
+      <c r="F16" s="11"/>
+      <c r="G16" s="10">
         <f>IF(F16="","",EDATE(F16,12))</f>
       </c>
-      <c r="I16" s="7">
+      <c r="H16" s="11"/>
+      <c r="I16" s="10">
         <f>IF(H16="","",EDATE(H16,12))</f>
       </c>
-      <c r="K16" s="7">
+      <c r="J16" s="11"/>
+      <c r="K16" s="10">
         <f>IF(J16="","",EDATE(J16,36))</f>
       </c>
-      <c r="M16" s="7">
+      <c r="L16" s="11"/>
+      <c r="M16" s="10">
         <f>IF(L16="","",EDATE(L16,12))</f>
       </c>
-      <c r="O16" s="7">
+      <c r="N16" s="11"/>
+      <c r="O16" s="10">
         <f>IF(N16="","",EDATE(N16,12))</f>
       </c>
-      <c r="Q16" s="7">
+      <c r="P16" s="11"/>
+      <c r="Q16" s="10">
         <f>IF(P16="","",EDATE(P16,24))</f>
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="7">
+      <c r="A17" s="5"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="10">
         <f>IF(B17="","",EDATE(B17,12))</f>
       </c>
-      <c r="E17" s="7">
+      <c r="D17" s="11"/>
+      <c r="E17" s="10">
         <f>IF(D17="","",EDATE(D17,36))</f>
       </c>
-      <c r="G17" s="7">
+      <c r="F17" s="11"/>
+      <c r="G17" s="10">
         <f>IF(F17="","",EDATE(F17,12))</f>
       </c>
-      <c r="I17" s="7">
+      <c r="H17" s="11"/>
+      <c r="I17" s="10">
         <f>IF(H17="","",EDATE(H17,12))</f>
       </c>
-      <c r="K17" s="7">
+      <c r="J17" s="11"/>
+      <c r="K17" s="10">
         <f>IF(J17="","",EDATE(J17,36))</f>
       </c>
-      <c r="M17" s="7">
+      <c r="L17" s="11"/>
+      <c r="M17" s="10">
         <f>IF(L17="","",EDATE(L17,12))</f>
       </c>
-      <c r="O17" s="7">
+      <c r="N17" s="11"/>
+      <c r="O17" s="10">
         <f>IF(N17="","",EDATE(N17,12))</f>
       </c>
-      <c r="Q17" s="7">
+      <c r="P17" s="11"/>
+      <c r="Q17" s="10">
         <f>IF(P17="","",EDATE(P17,24))</f>
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="7">
+      <c r="A18" s="5"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="10">
         <f>IF(B18="","",EDATE(B18,12))</f>
       </c>
-      <c r="E18" s="7">
+      <c r="D18" s="11"/>
+      <c r="E18" s="10">
         <f>IF(D18="","",EDATE(D18,36))</f>
       </c>
-      <c r="G18" s="7">
+      <c r="F18" s="11"/>
+      <c r="G18" s="10">
         <f>IF(F18="","",EDATE(F18,12))</f>
       </c>
-      <c r="I18" s="7">
+      <c r="H18" s="11"/>
+      <c r="I18" s="10">
         <f>IF(H18="","",EDATE(H18,12))</f>
       </c>
-      <c r="K18" s="7">
+      <c r="J18" s="11"/>
+      <c r="K18" s="10">
         <f>IF(J18="","",EDATE(J18,36))</f>
       </c>
-      <c r="M18" s="7">
+      <c r="L18" s="11"/>
+      <c r="M18" s="10">
         <f>IF(L18="","",EDATE(L18,12))</f>
       </c>
-      <c r="O18" s="7">
+      <c r="N18" s="11"/>
+      <c r="O18" s="10">
         <f>IF(N18="","",EDATE(N18,12))</f>
       </c>
-      <c r="Q18" s="7">
+      <c r="P18" s="11"/>
+      <c r="Q18" s="10">
         <f>IF(P18="","",EDATE(P18,24))</f>
       </c>
     </row>
     <row r="19">
-      <c r="C19" s="7">
+      <c r="A19" s="5"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="10">
         <f>IF(B19="","",EDATE(B19,12))</f>
       </c>
-      <c r="E19" s="7">
+      <c r="D19" s="11"/>
+      <c r="E19" s="10">
         <f>IF(D19="","",EDATE(D19,36))</f>
       </c>
-      <c r="G19" s="7">
+      <c r="F19" s="11"/>
+      <c r="G19" s="10">
         <f>IF(F19="","",EDATE(F19,12))</f>
       </c>
-      <c r="I19" s="7">
+      <c r="H19" s="11"/>
+      <c r="I19" s="10">
         <f>IF(H19="","",EDATE(H19,12))</f>
       </c>
-      <c r="K19" s="7">
+      <c r="J19" s="11"/>
+      <c r="K19" s="10">
         <f>IF(J19="","",EDATE(J19,36))</f>
       </c>
-      <c r="M19" s="7">
+      <c r="L19" s="11"/>
+      <c r="M19" s="10">
         <f>IF(L19="","",EDATE(L19,12))</f>
       </c>
-      <c r="O19" s="7">
+      <c r="N19" s="11"/>
+      <c r="O19" s="10">
         <f>IF(N19="","",EDATE(N19,12))</f>
       </c>
-      <c r="Q19" s="7">
+      <c r="P19" s="11"/>
+      <c r="Q19" s="10">
         <f>IF(P19="","",EDATE(P19,24))</f>
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="7">
+      <c r="A20" s="5"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="10">
         <f>IF(B20="","",EDATE(B20,12))</f>
       </c>
-      <c r="E20" s="7">
+      <c r="D20" s="11"/>
+      <c r="E20" s="10">
         <f>IF(D20="","",EDATE(D20,36))</f>
       </c>
-      <c r="G20" s="7">
+      <c r="F20" s="11"/>
+      <c r="G20" s="10">
         <f>IF(F20="","",EDATE(F20,12))</f>
       </c>
-      <c r="I20" s="7">
+      <c r="H20" s="11"/>
+      <c r="I20" s="10">
         <f>IF(H20="","",EDATE(H20,12))</f>
       </c>
-      <c r="K20" s="7">
+      <c r="J20" s="11"/>
+      <c r="K20" s="10">
         <f>IF(J20="","",EDATE(J20,36))</f>
       </c>
-      <c r="M20" s="7">
+      <c r="L20" s="11"/>
+      <c r="M20" s="10">
         <f>IF(L20="","",EDATE(L20,12))</f>
       </c>
-      <c r="O20" s="7">
+      <c r="N20" s="11"/>
+      <c r="O20" s="10">
         <f>IF(N20="","",EDATE(N20,12))</f>
       </c>
-      <c r="Q20" s="7">
+      <c r="P20" s="11"/>
+      <c r="Q20" s="10">
         <f>IF(P20="","",EDATE(P20,24))</f>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="7">
+      <c r="A21" s="5"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="10">
         <f>IF(B21="","",EDATE(B21,12))</f>
       </c>
-      <c r="E21" s="7">
+      <c r="D21" s="11"/>
+      <c r="E21" s="10">
         <f>IF(D21="","",EDATE(D21,36))</f>
       </c>
-      <c r="G21" s="7">
+      <c r="F21" s="11"/>
+      <c r="G21" s="10">
         <f>IF(F21="","",EDATE(F21,12))</f>
       </c>
-      <c r="I21" s="7">
+      <c r="H21" s="11"/>
+      <c r="I21" s="10">
         <f>IF(H21="","",EDATE(H21,12))</f>
       </c>
-      <c r="K21" s="7">
+      <c r="J21" s="11"/>
+      <c r="K21" s="10">
         <f>IF(J21="","",EDATE(J21,36))</f>
       </c>
-      <c r="M21" s="7">
+      <c r="L21" s="11"/>
+      <c r="M21" s="10">
         <f>IF(L21="","",EDATE(L21,12))</f>
       </c>
-      <c r="O21" s="7">
+      <c r="N21" s="11"/>
+      <c r="O21" s="10">
         <f>IF(N21="","",EDATE(N21,12))</f>
       </c>
-      <c r="Q21" s="7">
+      <c r="P21" s="11"/>
+      <c r="Q21" s="10">
         <f>IF(P21="","",EDATE(P21,24))</f>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="7">
+      <c r="A22" s="5"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="10">
         <f>IF(B22="","",EDATE(B22,12))</f>
       </c>
-      <c r="E22" s="7">
+      <c r="D22" s="11"/>
+      <c r="E22" s="10">
         <f>IF(D22="","",EDATE(D22,36))</f>
       </c>
-      <c r="G22" s="7">
+      <c r="F22" s="11"/>
+      <c r="G22" s="10">
         <f>IF(F22="","",EDATE(F22,12))</f>
       </c>
-      <c r="I22" s="7">
+      <c r="H22" s="11"/>
+      <c r="I22" s="10">
         <f>IF(H22="","",EDATE(H22,12))</f>
       </c>
-      <c r="K22" s="7">
+      <c r="J22" s="11"/>
+      <c r="K22" s="10">
         <f>IF(J22="","",EDATE(J22,36))</f>
       </c>
-      <c r="M22" s="7">
+      <c r="L22" s="11"/>
+      <c r="M22" s="10">
         <f>IF(L22="","",EDATE(L22,12))</f>
       </c>
-      <c r="O22" s="7">
+      <c r="N22" s="11"/>
+      <c r="O22" s="10">
         <f>IF(N22="","",EDATE(N22,12))</f>
       </c>
-      <c r="Q22" s="7">
+      <c r="P22" s="11"/>
+      <c r="Q22" s="10">
         <f>IF(P22="","",EDATE(P22,24))</f>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="7">
+      <c r="A23" s="5"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="10">
         <f>IF(B23="","",EDATE(B23,12))</f>
       </c>
-      <c r="E23" s="7">
+      <c r="D23" s="11"/>
+      <c r="E23" s="10">
         <f>IF(D23="","",EDATE(D23,36))</f>
       </c>
-      <c r="G23" s="7">
+      <c r="F23" s="11"/>
+      <c r="G23" s="10">
         <f>IF(F23="","",EDATE(F23,12))</f>
       </c>
-      <c r="I23" s="7">
+      <c r="H23" s="11"/>
+      <c r="I23" s="10">
         <f>IF(H23="","",EDATE(H23,12))</f>
       </c>
-      <c r="K23" s="7">
+      <c r="J23" s="11"/>
+      <c r="K23" s="10">
         <f>IF(J23="","",EDATE(J23,36))</f>
       </c>
-      <c r="M23" s="7">
+      <c r="L23" s="11"/>
+      <c r="M23" s="10">
         <f>IF(L23="","",EDATE(L23,12))</f>
       </c>
-      <c r="O23" s="7">
+      <c r="N23" s="11"/>
+      <c r="O23" s="10">
         <f>IF(N23="","",EDATE(N23,12))</f>
       </c>
-      <c r="Q23" s="7">
+      <c r="P23" s="11"/>
+      <c r="Q23" s="10">
         <f>IF(P23="","",EDATE(P23,24))</f>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="7">
+      <c r="A24" s="5"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="10">
         <f>IF(B24="","",EDATE(B24,12))</f>
       </c>
-      <c r="E24" s="7">
+      <c r="D24" s="11"/>
+      <c r="E24" s="10">
         <f>IF(D24="","",EDATE(D24,36))</f>
       </c>
-      <c r="G24" s="7">
+      <c r="F24" s="11"/>
+      <c r="G24" s="10">
         <f>IF(F24="","",EDATE(F24,12))</f>
       </c>
-      <c r="I24" s="7">
+      <c r="H24" s="11"/>
+      <c r="I24" s="10">
         <f>IF(H24="","",EDATE(H24,12))</f>
       </c>
-      <c r="K24" s="7">
+      <c r="J24" s="11"/>
+      <c r="K24" s="10">
         <f>IF(J24="","",EDATE(J24,36))</f>
       </c>
-      <c r="M24" s="7">
+      <c r="L24" s="11"/>
+      <c r="M24" s="10">
         <f>IF(L24="","",EDATE(L24,12))</f>
       </c>
-      <c r="O24" s="7">
+      <c r="N24" s="11"/>
+      <c r="O24" s="10">
         <f>IF(N24="","",EDATE(N24,12))</f>
       </c>
-      <c r="Q24" s="7">
+      <c r="P24" s="11"/>
+      <c r="Q24" s="10">
         <f>IF(P24="","",EDATE(P24,24))</f>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="7">
+      <c r="A25" s="5"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="10">
         <f>IF(B25="","",EDATE(B25,12))</f>
       </c>
-      <c r="E25" s="7">
+      <c r="D25" s="11"/>
+      <c r="E25" s="10">
         <f>IF(D25="","",EDATE(D25,36))</f>
       </c>
-      <c r="G25" s="7">
+      <c r="F25" s="11"/>
+      <c r="G25" s="10">
         <f>IF(F25="","",EDATE(F25,12))</f>
       </c>
-      <c r="I25" s="7">
+      <c r="H25" s="11"/>
+      <c r="I25" s="10">
         <f>IF(H25="","",EDATE(H25,12))</f>
       </c>
-      <c r="K25" s="7">
+      <c r="J25" s="11"/>
+      <c r="K25" s="10">
         <f>IF(J25="","",EDATE(J25,36))</f>
       </c>
-      <c r="M25" s="7">
+      <c r="L25" s="11"/>
+      <c r="M25" s="10">
         <f>IF(L25="","",EDATE(L25,12))</f>
       </c>
-      <c r="O25" s="7">
+      <c r="N25" s="11"/>
+      <c r="O25" s="10">
         <f>IF(N25="","",EDATE(N25,12))</f>
       </c>
-      <c r="Q25" s="7">
+      <c r="P25" s="11"/>
+      <c r="Q25" s="10">
         <f>IF(P25="","",EDATE(P25,24))</f>
       </c>
     </row>
     <row r="26">
-      <c r="C26" s="7">
+      <c r="A26" s="5"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="10">
         <f>IF(B26="","",EDATE(B26,12))</f>
       </c>
-      <c r="E26" s="7">
+      <c r="D26" s="11"/>
+      <c r="E26" s="10">
         <f>IF(D26="","",EDATE(D26,36))</f>
       </c>
-      <c r="G26" s="7">
+      <c r="F26" s="11"/>
+      <c r="G26" s="10">
         <f>IF(F26="","",EDATE(F26,12))</f>
       </c>
-      <c r="I26" s="7">
+      <c r="H26" s="11"/>
+      <c r="I26" s="10">
         <f>IF(H26="","",EDATE(H26,12))</f>
       </c>
-      <c r="K26" s="7">
+      <c r="J26" s="11"/>
+      <c r="K26" s="10">
         <f>IF(J26="","",EDATE(J26,36))</f>
       </c>
-      <c r="M26" s="7">
+      <c r="L26" s="11"/>
+      <c r="M26" s="10">
         <f>IF(L26="","",EDATE(L26,12))</f>
       </c>
-      <c r="O26" s="7">
+      <c r="N26" s="11"/>
+      <c r="O26" s="10">
         <f>IF(N26="","",EDATE(N26,12))</f>
       </c>
-      <c r="Q26" s="7">
+      <c r="P26" s="11"/>
+      <c r="Q26" s="10">
         <f>IF(P26="","",EDATE(P26,24))</f>
       </c>
     </row>
@@ -1179,7 +1389,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Name, your cycle in days (28 is common), and the date of the last supervision. The rest computes itself. The manager goes on this list too: theirs is the record inspectors ask for first.</t>
+          <t>Name, your cycle in days (28 is common), and the date of the last supervision. The tinted columns compute themselves. The manager goes on this list too.</t>
         </is>
       </c>
     </row>
@@ -1212,241 +1422,241 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Example: change or delete this row</t>
-        </is>
-      </c>
-      <c r="B5" s="8">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Example, overtype or delete me</t>
+        </is>
+      </c>
+      <c r="B5" s="11">
         <v>28</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="9">
         <v>46219</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="12">
         <f>IF(C5="","",TODAY()-C5)</f>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="12">
         <f>IF(C5="","",IF(TODAY()-C5&gt;B5,"OVERDUE",IF(TODAY()-C5&gt;B5-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="8">
-        <v>28</v>
-      </c>
-      <c r="D6" s="8">
+      <c r="A6" s="5"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12">
         <f>IF(C6="","",TODAY()-C6)</f>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="12">
         <f>IF(C6="","",IF(TODAY()-C6&gt;B6,"OVERDUE",IF(TODAY()-C6&gt;B6-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8">
-        <v>28</v>
-      </c>
-      <c r="D7" s="8">
+      <c r="A7" s="5"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="12">
         <f>IF(C7="","",TODAY()-C7)</f>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="12">
         <f>IF(C7="","",IF(TODAY()-C7&gt;B7,"OVERDUE",IF(TODAY()-C7&gt;B7-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="8">
-        <v>28</v>
-      </c>
-      <c r="D8" s="8">
+      <c r="A8" s="5"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="12">
         <f>IF(C8="","",TODAY()-C8)</f>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="12">
         <f>IF(C8="","",IF(TODAY()-C8&gt;B8,"OVERDUE",IF(TODAY()-C8&gt;B8-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="8">
-        <v>28</v>
-      </c>
-      <c r="D9" s="8">
+      <c r="A9" s="5"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="12">
         <f>IF(C9="","",TODAY()-C9)</f>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="12">
         <f>IF(C9="","",IF(TODAY()-C9&gt;B9,"OVERDUE",IF(TODAY()-C9&gt;B9-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="8">
-        <v>28</v>
-      </c>
-      <c r="D10" s="8">
+      <c r="A10" s="5"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="12">
         <f>IF(C10="","",TODAY()-C10)</f>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="12">
         <f>IF(C10="","",IF(TODAY()-C10&gt;B10,"OVERDUE",IF(TODAY()-C10&gt;B10-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="8">
-        <v>28</v>
-      </c>
-      <c r="D11" s="8">
+      <c r="A11" s="5"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="12">
         <f>IF(C11="","",TODAY()-C11)</f>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="12">
         <f>IF(C11="","",IF(TODAY()-C11&gt;B11,"OVERDUE",IF(TODAY()-C11&gt;B11-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="8">
-        <v>28</v>
-      </c>
-      <c r="D12" s="8">
+      <c r="A12" s="5"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="12">
         <f>IF(C12="","",TODAY()-C12)</f>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="12">
         <f>IF(C12="","",IF(TODAY()-C12&gt;B12,"OVERDUE",IF(TODAY()-C12&gt;B12-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="8">
-        <v>28</v>
-      </c>
-      <c r="D13" s="8">
+      <c r="A13" s="5"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="12">
         <f>IF(C13="","",TODAY()-C13)</f>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="12">
         <f>IF(C13="","",IF(TODAY()-C13&gt;B13,"OVERDUE",IF(TODAY()-C13&gt;B13-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="8">
-        <v>28</v>
-      </c>
-      <c r="D14" s="8">
+      <c r="A14" s="5"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="12">
         <f>IF(C14="","",TODAY()-C14)</f>
       </c>
-      <c r="E14" s="8">
+      <c r="E14" s="12">
         <f>IF(C14="","",IF(TODAY()-C14&gt;B14,"OVERDUE",IF(TODAY()-C14&gt;B14-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="8">
-        <v>28</v>
-      </c>
-      <c r="D15" s="8">
+      <c r="A15" s="5"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="12">
         <f>IF(C15="","",TODAY()-C15)</f>
       </c>
-      <c r="E15" s="8">
+      <c r="E15" s="12">
         <f>IF(C15="","",IF(TODAY()-C15&gt;B15,"OVERDUE",IF(TODAY()-C15&gt;B15-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="8">
-        <v>28</v>
-      </c>
-      <c r="D16" s="8">
+      <c r="A16" s="5"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="12">
         <f>IF(C16="","",TODAY()-C16)</f>
       </c>
-      <c r="E16" s="8">
+      <c r="E16" s="12">
         <f>IF(C16="","",IF(TODAY()-C16&gt;B16,"OVERDUE",IF(TODAY()-C16&gt;B16-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="8">
-        <v>28</v>
-      </c>
-      <c r="D17" s="8">
+      <c r="A17" s="5"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="12">
         <f>IF(C17="","",TODAY()-C17)</f>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="12">
         <f>IF(C17="","",IF(TODAY()-C17&gt;B17,"OVERDUE",IF(TODAY()-C17&gt;B17-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="8">
-        <v>28</v>
-      </c>
-      <c r="D18" s="8">
+      <c r="A18" s="5"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="12">
         <f>IF(C18="","",TODAY()-C18)</f>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="12">
         <f>IF(C18="","",IF(TODAY()-C18&gt;B18,"OVERDUE",IF(TODAY()-C18&gt;B18-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="8">
-        <v>28</v>
-      </c>
-      <c r="D19" s="8">
+      <c r="A19" s="5"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="12">
         <f>IF(C19="","",TODAY()-C19)</f>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="12">
         <f>IF(C19="","",IF(TODAY()-C19&gt;B19,"OVERDUE",IF(TODAY()-C19&gt;B19-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="8">
-        <v>28</v>
-      </c>
-      <c r="D20" s="8">
+      <c r="A20" s="5"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="12">
         <f>IF(C20="","",TODAY()-C20)</f>
       </c>
-      <c r="E20" s="8">
+      <c r="E20" s="12">
         <f>IF(C20="","",IF(TODAY()-C20&gt;B20,"OVERDUE",IF(TODAY()-C20&gt;B20-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="8">
-        <v>28</v>
-      </c>
-      <c r="D21" s="8">
+      <c r="A21" s="5"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="12">
         <f>IF(C21="","",TODAY()-C21)</f>
       </c>
-      <c r="E21" s="8">
+      <c r="E21" s="12">
         <f>IF(C21="","",IF(TODAY()-C21&gt;B21,"OVERDUE",IF(TODAY()-C21&gt;B21-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="8">
-        <v>28</v>
-      </c>
-      <c r="D22" s="8">
+      <c r="A22" s="5"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="12">
         <f>IF(C22="","",TODAY()-C22)</f>
       </c>
-      <c r="E22" s="8">
+      <c r="E22" s="12">
         <f>IF(C22="","",IF(TODAY()-C22&gt;B22,"OVERDUE",IF(TODAY()-C22&gt;B22-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="8">
-        <v>28</v>
-      </c>
-      <c r="D23" s="8">
+      <c r="A23" s="5"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="12">
         <f>IF(C23="","",TODAY()-C23)</f>
       </c>
-      <c r="E23" s="8">
+      <c r="E23" s="12">
         <f>IF(C23="","",IF(TODAY()-C23&gt;B23,"OVERDUE",IF(TODAY()-C23&gt;B23-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="8">
-        <v>28</v>
-      </c>
-      <c r="D24" s="8">
+      <c r="A24" s="5"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="12">
         <f>IF(C24="","",TODAY()-C24)</f>
       </c>
-      <c r="E24" s="8">
+      <c r="E24" s="12">
         <f>IF(C24="","",IF(TODAY()-C24&gt;B24,"OVERDUE",IF(TODAY()-C24&gt;B24-7,"DUE","OK")))</f>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="8">
-        <v>28</v>
-      </c>
-      <c r="D25" s="8">
+      <c r="A25" s="5"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="12">
         <f>IF(C25="","",TODAY()-C25)</f>
       </c>
-      <c r="E25" s="8">
+      <c r="E25" s="12">
         <f>IF(C25="","",IF(TODAY()-C25&gt;B25,"OVERDUE",IF(TODAY()-C25&gt;B25-7,"DUE","OK")))</f>
       </c>
     </row>
@@ -1497,7 +1707,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>For staff on the Update Service: run the status check twice a year (one minute each, with consent) and note the date. Next due computes itself. "When did you last check?" is a real inspection question.</t>
+          <t>For staff on the Update Service: run the status check twice a year (one minute each, with consent) and note the date. Next due computes itself.</t>
         </is>
       </c>
     </row>
@@ -1535,132 +1745,232 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Example: change or delete this row</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Example, overtype or delete me</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>001234567890</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <v>46059</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="10">
         <f>IF(D5="","",EDATE(D5,6))</f>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>No change</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="E6" s="7">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="10">
         <f>IF(D6="","",EDATE(D6,6))</f>
       </c>
+      <c r="F6" s="5"/>
     </row>
     <row r="7">
-      <c r="E7" s="7">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="10">
         <f>IF(D7="","",EDATE(D7,6))</f>
       </c>
+      <c r="F7" s="5"/>
     </row>
     <row r="8">
-      <c r="E8" s="7">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="10">
         <f>IF(D8="","",EDATE(D8,6))</f>
       </c>
+      <c r="F8" s="5"/>
     </row>
     <row r="9">
-      <c r="E9" s="7">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="10">
         <f>IF(D9="","",EDATE(D9,6))</f>
       </c>
+      <c r="F9" s="5"/>
     </row>
     <row r="10">
-      <c r="E10" s="7">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="10">
         <f>IF(D10="","",EDATE(D10,6))</f>
       </c>
+      <c r="F10" s="5"/>
     </row>
     <row r="11">
-      <c r="E11" s="7">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="10">
         <f>IF(D11="","",EDATE(D11,6))</f>
       </c>
+      <c r="F11" s="5"/>
     </row>
     <row r="12">
-      <c r="E12" s="7">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="10">
         <f>IF(D12="","",EDATE(D12,6))</f>
       </c>
+      <c r="F12" s="5"/>
     </row>
     <row r="13">
-      <c r="E13" s="7">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="10">
         <f>IF(D13="","",EDATE(D13,6))</f>
       </c>
+      <c r="F13" s="5"/>
     </row>
     <row r="14">
-      <c r="E14" s="7">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="10">
         <f>IF(D14="","",EDATE(D14,6))</f>
       </c>
+      <c r="F14" s="5"/>
     </row>
     <row r="15">
-      <c r="E15" s="7">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="10">
         <f>IF(D15="","",EDATE(D15,6))</f>
       </c>
+      <c r="F15" s="5"/>
     </row>
     <row r="16">
-      <c r="E16" s="7">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="10">
         <f>IF(D16="","",EDATE(D16,6))</f>
       </c>
+      <c r="F16" s="5"/>
     </row>
     <row r="17">
-      <c r="E17" s="7">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="10">
         <f>IF(D17="","",EDATE(D17,6))</f>
       </c>
+      <c r="F17" s="5"/>
     </row>
     <row r="18">
-      <c r="E18" s="7">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="10">
         <f>IF(D18="","",EDATE(D18,6))</f>
       </c>
+      <c r="F18" s="5"/>
     </row>
     <row r="19">
-      <c r="E19" s="7">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="10">
         <f>IF(D19="","",EDATE(D19,6))</f>
       </c>
+      <c r="F19" s="5"/>
     </row>
     <row r="20">
-      <c r="E20" s="7">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="10">
         <f>IF(D20="","",EDATE(D20,6))</f>
       </c>
+      <c r="F20" s="5"/>
     </row>
     <row r="21">
-      <c r="E21" s="7">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="10">
         <f>IF(D21="","",EDATE(D21,6))</f>
       </c>
+      <c r="F21" s="5"/>
     </row>
     <row r="22">
-      <c r="E22" s="7">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="10">
         <f>IF(D22="","",EDATE(D22,6))</f>
       </c>
+      <c r="F22" s="5"/>
     </row>
     <row r="23">
-      <c r="E23" s="7">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="10">
         <f>IF(D23="","",EDATE(D23,6))</f>
       </c>
+      <c r="F23" s="5"/>
     </row>
     <row r="24">
-      <c r="E24" s="7">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="10">
         <f>IF(D24="","",EDATE(D24,6))</f>
       </c>
+      <c r="F24" s="5"/>
     </row>
     <row r="25">
-      <c r="E25" s="7">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="10">
         <f>IF(D25="","",EDATE(D25,6))</f>
       </c>
+      <c r="F25" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1707,7 +2017,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Care staff must gain the Level 3 Diploma within two years of starting. Type their start date and whether they hold it; the deadline computes itself and goes red when it passes.</t>
+          <t>Care staff must gain the Level 3 Diploma within two years of starting. Start date plus Yes or No; the deadline computes itself.</t>
         </is>
       </c>
     </row>
@@ -1735,140 +2045,180 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Example: change or delete this row</t>
-        </is>
-      </c>
-      <c r="B5" s="7">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Example, overtype or delete me</t>
+        </is>
+      </c>
+      <c r="B5" s="9">
         <v>45759</v>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="10">
         <f>IF(OR(B5="",C5="Yes"),"",EDATE(B5,24))</f>
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="8"/>
-      <c r="D6" s="7">
+      <c r="A6" s="5"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="10">
         <f>IF(OR(B6="",C6="Yes"),"",EDATE(B6,24))</f>
       </c>
     </row>
     <row r="7">
-      <c r="C7" s="8"/>
-      <c r="D7" s="7">
+      <c r="A7" s="5"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="10">
         <f>IF(OR(B7="",C7="Yes"),"",EDATE(B7,24))</f>
       </c>
     </row>
     <row r="8">
-      <c r="C8" s="8"/>
-      <c r="D8" s="7">
+      <c r="A8" s="5"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="10">
         <f>IF(OR(B8="",C8="Yes"),"",EDATE(B8,24))</f>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="8"/>
-      <c r="D9" s="7">
+      <c r="A9" s="5"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="10">
         <f>IF(OR(B9="",C9="Yes"),"",EDATE(B9,24))</f>
       </c>
     </row>
     <row r="10">
-      <c r="C10" s="8"/>
-      <c r="D10" s="7">
+      <c r="A10" s="5"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="10">
         <f>IF(OR(B10="",C10="Yes"),"",EDATE(B10,24))</f>
       </c>
     </row>
     <row r="11">
-      <c r="C11" s="8"/>
-      <c r="D11" s="7">
+      <c r="A11" s="5"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="10">
         <f>IF(OR(B11="",C11="Yes"),"",EDATE(B11,24))</f>
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="8"/>
-      <c r="D12" s="7">
+      <c r="A12" s="5"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="10">
         <f>IF(OR(B12="",C12="Yes"),"",EDATE(B12,24))</f>
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="8"/>
-      <c r="D13" s="7">
+      <c r="A13" s="5"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="10">
         <f>IF(OR(B13="",C13="Yes"),"",EDATE(B13,24))</f>
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="8"/>
-      <c r="D14" s="7">
+      <c r="A14" s="5"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="10">
         <f>IF(OR(B14="",C14="Yes"),"",EDATE(B14,24))</f>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="8"/>
-      <c r="D15" s="7">
+      <c r="A15" s="5"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="10">
         <f>IF(OR(B15="",C15="Yes"),"",EDATE(B15,24))</f>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="8"/>
-      <c r="D16" s="7">
+      <c r="A16" s="5"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="10">
         <f>IF(OR(B16="",C16="Yes"),"",EDATE(B16,24))</f>
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="8"/>
-      <c r="D17" s="7">
+      <c r="A17" s="5"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="10">
         <f>IF(OR(B17="",C17="Yes"),"",EDATE(B17,24))</f>
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="8"/>
-      <c r="D18" s="7">
+      <c r="A18" s="5"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="10">
         <f>IF(OR(B18="",C18="Yes"),"",EDATE(B18,24))</f>
       </c>
     </row>
     <row r="19">
-      <c r="C19" s="8"/>
-      <c r="D19" s="7">
+      <c r="A19" s="5"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="10">
         <f>IF(OR(B19="",C19="Yes"),"",EDATE(B19,24))</f>
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="8"/>
-      <c r="D20" s="7">
+      <c r="A20" s="5"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="10">
         <f>IF(OR(B20="",C20="Yes"),"",EDATE(B20,24))</f>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="8"/>
-      <c r="D21" s="7">
+      <c r="A21" s="5"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="10">
         <f>IF(OR(B21="",C21="Yes"),"",EDATE(B21,24))</f>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="8"/>
-      <c r="D22" s="7">
+      <c r="A22" s="5"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="10">
         <f>IF(OR(B22="",C22="Yes"),"",EDATE(B22,24))</f>
       </c>
     </row>
     <row r="23">
-      <c r="C23" s="8"/>
-      <c r="D23" s="7">
+      <c r="A23" s="5"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="10">
         <f>IF(OR(B23="",C23="Yes"),"",EDATE(B23,24))</f>
       </c>
     </row>
     <row r="24">
-      <c r="C24" s="8"/>
-      <c r="D24" s="7">
+      <c r="A24" s="5"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="10">
         <f>IF(OR(B24="",C24="Yes"),"",EDATE(B24,24))</f>
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="8"/>
-      <c r="D25" s="7">
+      <c r="A25" s="5"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="10">
         <f>IF(OR(B25="",C25="Yes"),"",EDATE(B25,24))</f>
       </c>
     </row>
@@ -1917,7 +2267,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The documents every home must keep under review. Type the date each was last reviewed; the next-due date computes itself. Below: the two visit clocks inspectors always check.</t>
+          <t>Type the date each document was last reviewed; the next-due date computes itself. Below: the monthly independent visit grid.</t>
         </is>
       </c>
     </row>
@@ -1945,106 +2295,114 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Statement of purpose</t>
         </is>
       </c>
-      <c r="C5" s="8">
+      <c r="B5" s="11"/>
+      <c r="C5" s="11">
         <v>12</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="10">
         <f>IF(B5="","",EDATE(B5,C5))</f>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Location risk assessment</t>
         </is>
       </c>
-      <c r="C6" s="8">
+      <c r="B6" s="11"/>
+      <c r="C6" s="11">
         <v>12</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="10">
         <f>IF(B6="","",EDATE(B6,C6))</f>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Safeguarding policy</t>
         </is>
       </c>
-      <c r="C7" s="8">
+      <c r="B7" s="11"/>
+      <c r="C7" s="11">
         <v>12</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="10">
         <f>IF(B7="","",EDATE(B7,C7))</f>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Behaviour support policy</t>
         </is>
       </c>
-      <c r="C8" s="8">
+      <c r="B8" s="11"/>
+      <c r="C8" s="11">
         <v>12</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="10">
         <f>IF(B8="","",EDATE(B8,C8))</f>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Missing child policy</t>
         </is>
       </c>
-      <c r="C9" s="8">
+      <c r="B9" s="11"/>
+      <c r="C9" s="11">
         <v>12</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="10">
         <f>IF(B9="","",EDATE(B9,C9))</f>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Complaints policy</t>
         </is>
       </c>
-      <c r="C10" s="8">
+      <c r="B10" s="11"/>
+      <c r="C10" s="11">
         <v>12</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="10">
         <f>IF(B10="","",EDATE(B10,C10))</f>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Lone working assessment</t>
         </is>
       </c>
-      <c r="C11" s="8">
+      <c r="B11" s="11"/>
+      <c r="C11" s="11">
         <v>12</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="10">
         <f>IF(B11="","",EDATE(B11,C11))</f>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Workforce plan</t>
         </is>
       </c>
-      <c r="C12" s="8">
+      <c r="B12" s="11"/>
+      <c r="C12" s="11">
         <v>12</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="10">
         <f>IF(B12="","",EDATE(B12,C12))</f>
       </c>
     </row>
@@ -2052,7 +2410,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>The two visit clocks</t>
+          <t>The monthly visit (regulation 44)</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2422,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Reg 44 visit date</t>
+          <t>Visit date</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -2079,92 +2437,128 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>January</t>
         </is>
       </c>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>February</t>
         </is>
       </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>March</t>
         </is>
       </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>April</t>
         </is>
       </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>July</t>
         </is>
       </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>September</t>
         </is>
       </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>October</t>
         </is>
       </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>November</t>
         </is>
       </c>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>December</t>
         </is>
       </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
     </row>
     <row r="28"/>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Reg 45 quality of care review: due every six months, sent to Ofsted within 28 days of completing it.</t>
         </is>
@@ -2249,139 +2643,154 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Proof of identity, with a recent photograph</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Passport or licence plus a dated photo, copies in the file</t>
         </is>
       </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Enhanced DBS with children's barred list check</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Certificate number and date recorded; never the disclosure content</t>
         </is>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Two written references, one from the most recent employer</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>On file, checked by phone, with a note of the call</t>
         </is>
       </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="5"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Why previous work with children or vulnerable adults ended</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Checked as far as practicable, in writing</t>
         </is>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Documentary evidence of qualifications</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>The certificates themselves, not a CV line</t>
         </is>
       </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Full employment history with every gap explained in writing</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Use the Employment gaps tab; anything over a month needs a sentence</t>
         </is>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Right to work in the UK</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Evidence checked and copied before day one</t>
         </is>
       </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Health: fit for the role</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Assessment date recorded; the assessment itself stays with occupational health</t>
         </is>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="5"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Interview record</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Who interviewed, when, and the judgment reached</t>
         </is>
       </c>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="5"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>DBS Update Service status, if subscribed</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Consent noted and the date of the last status check</t>
         </is>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2456,70 +2865,126 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="11"/>
+    </row>
     <row r="6">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-    </row>
-    <row r="7"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="11"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="11"/>
+    </row>
     <row r="8">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-    </row>
-    <row r="9"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="11"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="11"/>
+    </row>
     <row r="10">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-    </row>
-    <row r="11"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="11"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="11"/>
+    </row>
     <row r="12">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-    </row>
-    <row r="13"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="11"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="11"/>
+    </row>
     <row r="14">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-    </row>
-    <row r="15"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="11"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="11"/>
+    </row>
     <row r="16">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-    </row>
-    <row r="17"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="11"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="11"/>
+    </row>
     <row r="18">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-    </row>
-    <row r="19"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="11"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="11"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
@@ -2582,100 +3047,118 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Statement of purpose, current and reviewed</t>
         </is>
       </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Staff list with qualifications and planned qualification updates</t>
         </is>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="5"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Recruitment and vetting records, complete for every person</t>
         </is>
       </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="5"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Training records, mandatory courses in date</t>
         </is>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="5"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Supervision records, everyone in cycle including the manager</t>
         </is>
       </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="5"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Staffing rotas, planned and as actually worked</t>
         </is>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="5"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Allegations records, held securely with timescales evidenced</t>
         </is>
       </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="5"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Reports of monthly regulation 44 visits</t>
         </is>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="5"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Regulation 45 quality of care report, within six months</t>
         </is>
       </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="5"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Notifications made to Ofsted, with who else was told</t>
         </is>
       </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="5"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Location assessment, reviewed within the year</t>
         </is>
       </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="5"/>
     </row>
     <row r="16"/>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
         </is>

</xml_diff>

<commit_message>
Pack: strip the self-promotion, keep one quiet origin mark per file
The give should not keep tapping the reader on the shoulder. Removed
'Free from Staffbook, keep it, copy it, share it' from three workbook
tabs, the per-page playbook footer, and the audit PDF's ad line and
tagline. What remains: staffbook.co.uk once on the Start here tab, the
wordmark on the playbook cover and audit header.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pack/staffbook-staff-file-pack.xlsx
+++ b/pack/staffbook-staff-file-pack.xlsx
@@ -316,7 +316,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
+          <t>staffbook.co.uk</t>
         </is>
       </c>
     </row>
@@ -370,7 +370,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Type the name, then the date each course was done under "Done on". The tinted Expires cell beside it fills in by itself. Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
+          <t>Type the name, then the date each course was done under "Done on". The tinted Expires cell beside it fills in by itself.</t>
         </is>
       </c>
     </row>
@@ -520,19 +520,19 @@
         </is>
       </c>
       <c r="B6" s="9">
-        <v>45859</v>
+        <v>45862</v>
       </c>
       <c r="C6" s="10">
         <f>IF(B6="","",EDATE(B6,12))</f>
       </c>
       <c r="D6" s="9">
-        <v>45259</v>
+        <v>45261</v>
       </c>
       <c r="E6" s="10">
         <f>IF(D6="","",EDATE(D6,36))</f>
       </c>
       <c r="F6" s="9">
-        <v>45909</v>
+        <v>45912</v>
       </c>
       <c r="G6" s="10">
         <f>IF(F6="","",EDATE(F6,12))</f>
@@ -1431,7 +1431,7 @@
         <v>28</v>
       </c>
       <c r="C5" s="9">
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="D5" s="12">
         <f>IF(C5="","",TODAY()-C5)</f>
@@ -1761,7 +1761,7 @@
         </is>
       </c>
       <c r="D5" s="9">
-        <v>46059</v>
+        <v>46061</v>
       </c>
       <c r="E5" s="10">
         <f>IF(D5="","",EDATE(D5,6))</f>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="B5" s="9">
-        <v>45759</v>
+        <v>45762</v>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
@@ -3156,14 +3156,6 @@
       <c r="C15" s="11"/>
       <c r="D15" s="5"/>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Free from Staffbook (staffbook.co.uk). Keep it, copy it, share it with another home.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>

</xml_diff>